<commit_message>
email auto upload for luboil
</commit_message>
<xml_diff>
--- a/Aepms-backend/data/Engine_Performance_Data.xlsx
+++ b/Aepms-backend/data/Engine_Performance_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GOKUL\Desktop\Ozellar_project\Aepms-backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GOKUL\Desktop\WORKPLACE\Workplace\Aepms-backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA3AE40-7B43-445A-97BE-D9C2196EEDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1ED77D-5904-4AE2-A294-C4F5C92A510E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vessel_info" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2153" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2920" uniqueCount="247">
   <si>
     <t>hull_no</t>
   </si>
@@ -692,14 +692,109 @@
   </si>
   <si>
     <t>mcr_limit</t>
+  </si>
+  <si>
+    <t>SE5S50-0063</t>
+  </si>
+  <si>
+    <t>AMNS POLAR</t>
+  </si>
+  <si>
+    <t>SF080102</t>
+  </si>
+  <si>
+    <t>PZM</t>
+  </si>
+  <si>
+    <t>SANFU</t>
+  </si>
+  <si>
+    <t>MAN B&amp;W</t>
+  </si>
+  <si>
+    <t>kg/cm2</t>
+  </si>
+  <si>
+    <t>GCL SARASWATI</t>
+  </si>
+  <si>
+    <t>Messrs. NYK Line</t>
+  </si>
+  <si>
+    <t>Oshima Shipbuilding Co., Ltd.</t>
+  </si>
+  <si>
+    <t>Mitsubishi Heavy Industries, Ltd.</t>
+  </si>
+  <si>
+    <t>Mitsubishi 6UEC60LS II</t>
+  </si>
+  <si>
+    <t>6UEC60LS II (IMO-Nox Tier I)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>GCL FOS</t>
+  </si>
+  <si>
+    <t>6S70MC-C</t>
+  </si>
+  <si>
+    <t>MITSUI ENGINEERING &amp; SHIPBUILDING CO., LTD.</t>
+  </si>
+  <si>
+    <t>MESSRS. KOTOBUKI KAIUN CO., LTD.</t>
+  </si>
+  <si>
+    <t>AMNSI STALLION</t>
+  </si>
+  <si>
+    <t>BC8.2-2</t>
+  </si>
+  <si>
+    <t>Qingdao Beihai Shipbuilding Heavy Industry C</t>
+  </si>
+  <si>
+    <t>Hebei Ocean Shipping Co.,Ltd.</t>
+  </si>
+  <si>
+    <t>5RT-flex58T-D</t>
+  </si>
+  <si>
+    <t>DALIAN MARINE DIESEL CO.,LTD (DMD-WÄRTSILÄ)</t>
+  </si>
+  <si>
+    <t>AMNS TUFMAX</t>
+  </si>
+  <si>
+    <t>SF080103</t>
+  </si>
+  <si>
+    <t>Taizhou Sanfu Ship Engineering</t>
+  </si>
+  <si>
+    <t>5S50MC-C</t>
+  </si>
+  <si>
+    <t>STX Dalian Engine Co.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -733,13 +828,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -784,8 +882,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:BT1048569" totalsRowShown="0">
-  <autoFilter ref="A1:BT1048569" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:BT1048576" totalsRowShown="0">
+  <autoFilter ref="A1:BT1048576" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="72">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="performance_data_id (PK)"/>
     <tableColumn id="73" xr3:uid="{00000000-0010-0000-0200-000049000000}" name="engine_no (UNIQUE, NOT NULL)"/>
@@ -1216,7 +1314,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AB18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
@@ -1224,10 +1322,11 @@
     <col min="3" max="3" width="25.44140625" customWidth="1"/>
     <col min="4" max="4" width="31.21875" customWidth="1"/>
     <col min="5" max="5" width="16.88671875" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" customWidth="1"/>
-    <col min="8" max="8" width="15.77734375" customWidth="1"/>
-    <col min="9" max="9" width="14.21875" customWidth="1"/>
-    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="27.33203125" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" customWidth="1"/>
+    <col min="10" max="10" width="24.5546875" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
     <col min="12" max="12" width="21.21875" customWidth="1"/>
     <col min="13" max="13" width="23" customWidth="1"/>
@@ -1915,6 +2014,333 @@
       </c>
       <c r="Z9" t="s">
         <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>219</v>
+      </c>
+      <c r="C10">
+        <v>9521813</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="F10" t="s">
+        <v>221</v>
+      </c>
+      <c r="G10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H10" t="s">
+        <v>246</v>
+      </c>
+      <c r="I10" t="s">
+        <v>245</v>
+      </c>
+      <c r="J10" t="s">
+        <v>218</v>
+      </c>
+      <c r="K10">
+        <v>5</v>
+      </c>
+      <c r="M10" t="s">
+        <v>19</v>
+      </c>
+      <c r="N10">
+        <v>168.37</v>
+      </c>
+      <c r="O10" t="s">
+        <v>20</v>
+      </c>
+      <c r="P10">
+        <v>6570</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>21</v>
+      </c>
+      <c r="R10">
+        <v>127</v>
+      </c>
+      <c r="S10" t="s">
+        <v>22</v>
+      </c>
+      <c r="T10">
+        <v>5585</v>
+      </c>
+      <c r="Y10">
+        <v>100</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="D11" s="3"/>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="D12" s="3"/>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>236</v>
+      </c>
+      <c r="C13">
+        <v>9628910</v>
+      </c>
+      <c r="D13">
+        <v>774</v>
+      </c>
+      <c r="E13" t="s">
+        <v>237</v>
+      </c>
+      <c r="F13" t="s">
+        <v>239</v>
+      </c>
+      <c r="G13" t="s">
+        <v>238</v>
+      </c>
+      <c r="H13" t="s">
+        <v>241</v>
+      </c>
+      <c r="I13" t="s">
+        <v>240</v>
+      </c>
+      <c r="J13" t="s">
+        <v>240</v>
+      </c>
+      <c r="K13">
+        <v>5</v>
+      </c>
+      <c r="M13" t="s">
+        <v>19</v>
+      </c>
+      <c r="N13" t="s">
+        <v>231</v>
+      </c>
+      <c r="O13" t="s">
+        <v>20</v>
+      </c>
+      <c r="P13">
+        <v>9760</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>21</v>
+      </c>
+      <c r="R13">
+        <v>92.9</v>
+      </c>
+      <c r="S13" t="s">
+        <v>22</v>
+      </c>
+      <c r="T13" t="s">
+        <v>231</v>
+      </c>
+      <c r="U13" t="s">
+        <v>231</v>
+      </c>
+      <c r="V13" t="s">
+        <v>231</v>
+      </c>
+      <c r="W13" t="s">
+        <v>231</v>
+      </c>
+      <c r="X13" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>242</v>
+      </c>
+      <c r="C14">
+        <v>9486295</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G14" t="s">
+        <v>244</v>
+      </c>
+      <c r="H14" t="s">
+        <v>223</v>
+      </c>
+      <c r="I14" t="s">
+        <v>245</v>
+      </c>
+      <c r="J14" t="s">
+        <v>245</v>
+      </c>
+      <c r="K14">
+        <v>5</v>
+      </c>
+      <c r="M14" t="s">
+        <v>19</v>
+      </c>
+      <c r="N14">
+        <v>164.6</v>
+      </c>
+      <c r="O14" t="s">
+        <v>20</v>
+      </c>
+      <c r="P14">
+        <v>6570</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>21</v>
+      </c>
+      <c r="R14">
+        <v>127</v>
+      </c>
+      <c r="S14" t="s">
+        <v>22</v>
+      </c>
+      <c r="T14">
+        <v>5510</v>
+      </c>
+      <c r="U14">
+        <v>56</v>
+      </c>
+      <c r="V14">
+        <v>73</v>
+      </c>
+      <c r="W14" t="s">
+        <v>231</v>
+      </c>
+      <c r="X14" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="D15" s="3"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="D16" s="3"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>225</v>
+      </c>
+      <c r="C17">
+        <v>9644500</v>
+      </c>
+      <c r="D17" s="2">
+        <v>4078</v>
+      </c>
+      <c r="E17" s="2">
+        <v>10701</v>
+      </c>
+      <c r="F17" t="s">
+        <v>226</v>
+      </c>
+      <c r="G17" t="s">
+        <v>227</v>
+      </c>
+      <c r="H17" t="s">
+        <v>228</v>
+      </c>
+      <c r="I17" t="s">
+        <v>229</v>
+      </c>
+      <c r="J17" t="s">
+        <v>230</v>
+      </c>
+      <c r="K17">
+        <v>6</v>
+      </c>
+      <c r="M17" t="s">
+        <v>19</v>
+      </c>
+      <c r="N17">
+        <v>166.6</v>
+      </c>
+      <c r="O17" t="s">
+        <v>20</v>
+      </c>
+      <c r="P17" s="4">
+        <v>12270</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>21</v>
+      </c>
+      <c r="R17">
+        <v>105</v>
+      </c>
+      <c r="S17" t="s">
+        <v>22</v>
+      </c>
+      <c r="T17" s="4">
+        <v>10436</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>232</v>
+      </c>
+      <c r="C18">
+        <v>9532082</v>
+      </c>
+      <c r="D18">
+        <v>5933</v>
+      </c>
+      <c r="F18" t="s">
+        <v>235</v>
+      </c>
+      <c r="G18" t="s">
+        <v>234</v>
+      </c>
+      <c r="H18" t="s">
+        <v>210</v>
+      </c>
+      <c r="I18" t="s">
+        <v>233</v>
+      </c>
+      <c r="J18" t="s">
+        <v>233</v>
+      </c>
+      <c r="K18">
+        <v>6</v>
+      </c>
+      <c r="N18">
+        <v>163.69999999999999</v>
+      </c>
+      <c r="O18" t="s">
+        <v>20</v>
+      </c>
+      <c r="P18">
+        <v>16860</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>21</v>
+      </c>
+      <c r="R18">
+        <v>91</v>
+      </c>
+      <c r="S18" t="s">
+        <v>22</v>
+      </c>
+      <c r="T18">
+        <v>14330</v>
       </c>
     </row>
   </sheetData>
@@ -2332,7 +2758,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:BT54"/>
+  <dimension ref="A1:BT73"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="26.21875" customWidth="1"/>
@@ -13435,6 +13861,3435 @@
         <v>173</v>
       </c>
     </row>
+    <row r="55" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B55" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D55">
+        <v>25</v>
+      </c>
+      <c r="E55" t="s">
+        <v>171</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <v>1643</v>
+      </c>
+      <c r="H55" t="s">
+        <v>21</v>
+      </c>
+      <c r="I55">
+        <v>80</v>
+      </c>
+      <c r="J55" t="s">
+        <v>22</v>
+      </c>
+      <c r="K55">
+        <v>14</v>
+      </c>
+      <c r="L55" t="s">
+        <v>135</v>
+      </c>
+      <c r="M55">
+        <v>24</v>
+      </c>
+      <c r="N55" t="s">
+        <v>171</v>
+      </c>
+      <c r="O55">
+        <v>1023</v>
+      </c>
+      <c r="P55" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q55">
+        <v>17</v>
+      </c>
+      <c r="R55" t="s">
+        <v>135</v>
+      </c>
+      <c r="S55">
+        <v>35</v>
+      </c>
+      <c r="T55" t="s">
+        <v>135</v>
+      </c>
+      <c r="U55">
+        <v>40</v>
+      </c>
+      <c r="V55" t="s">
+        <v>173</v>
+      </c>
+      <c r="W55">
+        <v>75</v>
+      </c>
+      <c r="X55" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y55">
+        <v>52</v>
+      </c>
+      <c r="Z55" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA55">
+        <v>6.28</v>
+      </c>
+      <c r="AB55" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC55">
+        <v>34.200000000000003</v>
+      </c>
+      <c r="AD55" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE55">
+        <v>251</v>
+      </c>
+      <c r="AF55" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG55">
+        <v>295</v>
+      </c>
+      <c r="AH55" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI55">
+        <v>235</v>
+      </c>
+      <c r="AJ55" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK55">
+        <v>7</v>
+      </c>
+      <c r="AL55" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM55">
+        <v>0.35</v>
+      </c>
+      <c r="AN55" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO55">
+        <v>0.25</v>
+      </c>
+      <c r="AP55" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ55">
+        <v>26</v>
+      </c>
+      <c r="AR55" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS55">
+        <v>300</v>
+      </c>
+      <c r="AT55" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU55">
+        <v>182.59</v>
+      </c>
+      <c r="AV55" t="s">
+        <v>20</v>
+      </c>
+      <c r="BJ55">
+        <v>183.02</v>
+      </c>
+      <c r="BK55" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B56" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D56">
+        <v>50</v>
+      </c>
+      <c r="E56" t="s">
+        <v>171</v>
+      </c>
+      <c r="F56">
+        <v>2</v>
+      </c>
+      <c r="G56">
+        <v>3285</v>
+      </c>
+      <c r="H56" t="s">
+        <v>21</v>
+      </c>
+      <c r="I56">
+        <v>100.8</v>
+      </c>
+      <c r="J56" t="s">
+        <v>22</v>
+      </c>
+      <c r="K56">
+        <v>14</v>
+      </c>
+      <c r="L56" t="s">
+        <v>135</v>
+      </c>
+      <c r="M56">
+        <v>28</v>
+      </c>
+      <c r="N56" t="s">
+        <v>171</v>
+      </c>
+      <c r="O56">
+        <v>1023</v>
+      </c>
+      <c r="P56" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q56">
+        <v>17</v>
+      </c>
+      <c r="R56" t="s">
+        <v>135</v>
+      </c>
+      <c r="S56">
+        <v>30</v>
+      </c>
+      <c r="T56" t="s">
+        <v>135</v>
+      </c>
+      <c r="U56">
+        <v>90</v>
+      </c>
+      <c r="V56" t="s">
+        <v>173</v>
+      </c>
+      <c r="W56">
+        <v>105.2</v>
+      </c>
+      <c r="X56" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y56">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="Z56" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA56">
+        <v>9.9600000000000009</v>
+      </c>
+      <c r="AB56" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC56">
+        <v>46.2</v>
+      </c>
+      <c r="AD56" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE56">
+        <v>271</v>
+      </c>
+      <c r="AF56" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG56">
+        <v>325</v>
+      </c>
+      <c r="AH56" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI56">
+        <v>235</v>
+      </c>
+      <c r="AJ56" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK56">
+        <v>12.6</v>
+      </c>
+      <c r="AL56" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM56">
+        <v>1</v>
+      </c>
+      <c r="AN56" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO56">
+        <v>0.9</v>
+      </c>
+      <c r="AP56" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ56">
+        <v>26</v>
+      </c>
+      <c r="AR56" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS56">
+        <v>552</v>
+      </c>
+      <c r="AT56" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU56">
+        <v>168.04</v>
+      </c>
+      <c r="AV56" t="s">
+        <v>20</v>
+      </c>
+      <c r="BJ56">
+        <v>168.43</v>
+      </c>
+      <c r="BK56" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B57" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D57">
+        <v>75</v>
+      </c>
+      <c r="E57" t="s">
+        <v>171</v>
+      </c>
+      <c r="F57">
+        <v>3</v>
+      </c>
+      <c r="G57">
+        <v>4928</v>
+      </c>
+      <c r="H57" t="s">
+        <v>21</v>
+      </c>
+      <c r="I57">
+        <v>115.4</v>
+      </c>
+      <c r="J57" t="s">
+        <v>22</v>
+      </c>
+      <c r="K57">
+        <v>16</v>
+      </c>
+      <c r="L57" t="s">
+        <v>135</v>
+      </c>
+      <c r="M57">
+        <v>34</v>
+      </c>
+      <c r="N57" t="s">
+        <v>171</v>
+      </c>
+      <c r="O57">
+        <v>1022</v>
+      </c>
+      <c r="P57" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q57">
+        <v>18</v>
+      </c>
+      <c r="R57" t="s">
+        <v>135</v>
+      </c>
+      <c r="S57">
+        <v>30</v>
+      </c>
+      <c r="T57" t="s">
+        <v>135</v>
+      </c>
+      <c r="U57">
+        <v>126</v>
+      </c>
+      <c r="V57" t="s">
+        <v>173</v>
+      </c>
+      <c r="W57">
+        <v>142.80000000000001</v>
+      </c>
+      <c r="X57" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y57">
+        <v>113.4</v>
+      </c>
+      <c r="Z57" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA57">
+        <v>13.06</v>
+      </c>
+      <c r="AB57" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC57">
+        <v>56.4</v>
+      </c>
+      <c r="AD57" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE57">
+        <v>272</v>
+      </c>
+      <c r="AF57" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG57">
+        <v>330</v>
+      </c>
+      <c r="AH57" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI57">
+        <v>210</v>
+      </c>
+      <c r="AJ57" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK57">
+        <v>14.7</v>
+      </c>
+      <c r="AL57" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM57">
+        <v>1.75</v>
+      </c>
+      <c r="AN57" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO57">
+        <v>1.6</v>
+      </c>
+      <c r="AP57" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ57">
+        <v>26</v>
+      </c>
+      <c r="AR57" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS57">
+        <v>804</v>
+      </c>
+      <c r="AT57" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU57">
+        <v>163.15</v>
+      </c>
+      <c r="AV57" t="s">
+        <v>20</v>
+      </c>
+      <c r="BJ57">
+        <v>163.46</v>
+      </c>
+      <c r="BK57" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B58" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D58">
+        <v>85</v>
+      </c>
+      <c r="E58" t="s">
+        <v>171</v>
+      </c>
+      <c r="F58">
+        <v>4</v>
+      </c>
+      <c r="G58">
+        <v>5585</v>
+      </c>
+      <c r="H58" t="s">
+        <v>21</v>
+      </c>
+      <c r="I58">
+        <v>120.3</v>
+      </c>
+      <c r="J58" t="s">
+        <v>22</v>
+      </c>
+      <c r="K58">
+        <v>17</v>
+      </c>
+      <c r="L58" t="s">
+        <v>135</v>
+      </c>
+      <c r="M58">
+        <v>32</v>
+      </c>
+      <c r="N58" t="s">
+        <v>171</v>
+      </c>
+      <c r="O58">
+        <v>1021</v>
+      </c>
+      <c r="P58" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q58">
+        <v>18</v>
+      </c>
+      <c r="R58" t="s">
+        <v>135</v>
+      </c>
+      <c r="S58">
+        <v>36</v>
+      </c>
+      <c r="T58" t="s">
+        <v>135</v>
+      </c>
+      <c r="V58" t="s">
+        <v>173</v>
+      </c>
+      <c r="W58">
+        <v>152</v>
+      </c>
+      <c r="X58" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y58">
+        <v>124</v>
+      </c>
+      <c r="Z58" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA58">
+        <v>14.19</v>
+      </c>
+      <c r="AB58" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC58">
+        <v>60.4</v>
+      </c>
+      <c r="AD58" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE58">
+        <v>281</v>
+      </c>
+      <c r="AF58" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG58">
+        <v>345</v>
+      </c>
+      <c r="AH58" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI58">
+        <v>210</v>
+      </c>
+      <c r="AJ58" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK58">
+        <v>15.6</v>
+      </c>
+      <c r="AL58" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM58">
+        <v>2.15</v>
+      </c>
+      <c r="AN58" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO58">
+        <v>1.95</v>
+      </c>
+      <c r="AP58" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ58">
+        <v>28</v>
+      </c>
+      <c r="AR58" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS58">
+        <v>919.2</v>
+      </c>
+      <c r="AT58" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU58">
+        <v>164.58</v>
+      </c>
+      <c r="AV58" t="s">
+        <v>20</v>
+      </c>
+      <c r="BJ58">
+        <v>164.66</v>
+      </c>
+      <c r="BK58" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="59" spans="2:70" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D59" s="5">
+        <v>100</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="F59" s="5">
+        <v>5</v>
+      </c>
+      <c r="G59" s="5">
+        <v>6570</v>
+      </c>
+      <c r="H59" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I59" s="5">
+        <v>127</v>
+      </c>
+      <c r="J59" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K59" s="5">
+        <v>17</v>
+      </c>
+      <c r="L59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="M59" s="5">
+        <v>30</v>
+      </c>
+      <c r="N59" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="O59" s="5">
+        <v>1021</v>
+      </c>
+      <c r="P59" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q59" s="5">
+        <v>18</v>
+      </c>
+      <c r="R59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="S59" s="5">
+        <v>36</v>
+      </c>
+      <c r="T59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="U59" s="5">
+        <v>220</v>
+      </c>
+      <c r="V59" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="W59" s="5">
+        <v>151.80000000000001</v>
+      </c>
+      <c r="X59" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y59" s="5">
+        <v>148.19999999999999</v>
+      </c>
+      <c r="Z59" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA59" s="5">
+        <v>15.82</v>
+      </c>
+      <c r="AB59" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC59" s="5">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="AD59" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE59" s="5">
+        <v>293</v>
+      </c>
+      <c r="AF59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG59" s="5">
+        <v>375</v>
+      </c>
+      <c r="AH59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI59" s="5">
+        <v>220</v>
+      </c>
+      <c r="AJ59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK59" s="5">
+        <v>17</v>
+      </c>
+      <c r="AL59" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM59" s="5">
+        <v>2.7</v>
+      </c>
+      <c r="AN59" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO59" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="AP59" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ59" s="5">
+        <v>28</v>
+      </c>
+      <c r="AR59" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS59" s="5">
+        <v>1107</v>
+      </c>
+      <c r="AT59" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU59" s="5">
+        <v>168.49</v>
+      </c>
+      <c r="AV59" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="BJ59" s="5">
+        <v>168.37</v>
+      </c>
+      <c r="BK59" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="60" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B60" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D60">
+        <v>110</v>
+      </c>
+      <c r="E60" t="s">
+        <v>171</v>
+      </c>
+      <c r="F60">
+        <v>6</v>
+      </c>
+      <c r="G60">
+        <v>7227</v>
+      </c>
+      <c r="H60" t="s">
+        <v>21</v>
+      </c>
+      <c r="I60">
+        <v>131.1</v>
+      </c>
+      <c r="J60" t="s">
+        <v>22</v>
+      </c>
+      <c r="K60">
+        <v>17</v>
+      </c>
+      <c r="L60" t="s">
+        <v>135</v>
+      </c>
+      <c r="M60">
+        <v>26</v>
+      </c>
+      <c r="N60" t="s">
+        <v>171</v>
+      </c>
+      <c r="O60">
+        <v>1021</v>
+      </c>
+      <c r="P60" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q60">
+        <v>18</v>
+      </c>
+      <c r="R60" t="s">
+        <v>135</v>
+      </c>
+      <c r="S60">
+        <v>38</v>
+      </c>
+      <c r="T60" t="s">
+        <v>135</v>
+      </c>
+      <c r="U60">
+        <v>240</v>
+      </c>
+      <c r="V60" t="s">
+        <v>173</v>
+      </c>
+      <c r="W60">
+        <v>153.80000000000001</v>
+      </c>
+      <c r="X60" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y60">
+        <v>155.80000000000001</v>
+      </c>
+      <c r="Z60" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA60">
+        <v>16.850000000000001</v>
+      </c>
+      <c r="AB60" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC60">
+        <v>69.8</v>
+      </c>
+      <c r="AD60" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE60">
+        <v>304</v>
+      </c>
+      <c r="AF60" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG60">
+        <v>390</v>
+      </c>
+      <c r="AH60" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI60">
+        <v>220</v>
+      </c>
+      <c r="AJ60" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK60">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="AL60" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM60">
+        <v>2.85</v>
+      </c>
+      <c r="AN60" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO60">
+        <v>2.65</v>
+      </c>
+      <c r="AP60" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ60">
+        <v>29</v>
+      </c>
+      <c r="AR60" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS60">
+        <v>1236</v>
+      </c>
+      <c r="AT60" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU60">
+        <v>171.03</v>
+      </c>
+      <c r="AV60" t="s">
+        <v>20</v>
+      </c>
+      <c r="BJ60">
+        <v>170.8</v>
+      </c>
+      <c r="BK60" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B61" s="3"/>
+    </row>
+    <row r="62" spans="2:70" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B62" s="5">
+        <v>774</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D62" s="5">
+        <v>25</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="F62" s="5">
+        <v>1</v>
+      </c>
+      <c r="G62" s="5">
+        <v>2440</v>
+      </c>
+      <c r="H62" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I62" s="5">
+        <v>58</v>
+      </c>
+      <c r="J62" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K62" s="5">
+        <v>13</v>
+      </c>
+      <c r="L62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="M62" s="5">
+        <v>64</v>
+      </c>
+      <c r="N62" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="O62" s="5">
+        <v>1028</v>
+      </c>
+      <c r="P62" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q62" s="5">
+        <v>14.2</v>
+      </c>
+      <c r="R62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="S62" s="5">
+        <v>21</v>
+      </c>
+      <c r="T62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="U62" s="5">
+        <v>17</v>
+      </c>
+      <c r="V62" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="W62" s="5">
+        <v>80.2</v>
+      </c>
+      <c r="X62" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y62" s="5">
+        <v>50.6</v>
+      </c>
+      <c r="Z62" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA62" s="5">
+        <v>7.91</v>
+      </c>
+      <c r="AB62" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC62" s="5">
+        <v>29.5</v>
+      </c>
+      <c r="AD62" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE62" s="5">
+        <v>257</v>
+      </c>
+      <c r="AF62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG62" s="5">
+        <v>300</v>
+      </c>
+      <c r="AH62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI62" s="5">
+        <v>240</v>
+      </c>
+      <c r="AJ62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK62" s="5">
+        <v>6.35</v>
+      </c>
+      <c r="AL62" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM62" s="5">
+        <v>0.33</v>
+      </c>
+      <c r="AN62" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO62" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP62" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ62" s="5">
+        <v>18</v>
+      </c>
+      <c r="AR62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS62" s="5">
+        <v>434.78</v>
+      </c>
+      <c r="AT62" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU62" s="5">
+        <v>178.19</v>
+      </c>
+      <c r="AV62" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW62" s="5">
+        <v>77.5</v>
+      </c>
+      <c r="AX62" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY62" s="5">
+        <v>46.8</v>
+      </c>
+      <c r="AZ62" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA62" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB62" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC62" s="5">
+        <v>321.5</v>
+      </c>
+      <c r="BD62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE62" s="5">
+        <v>259.2</v>
+      </c>
+      <c r="BF62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG62" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH62" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI62" s="5">
+        <v>179.62</v>
+      </c>
+      <c r="BJ62" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK62" s="5">
+        <v>1000</v>
+      </c>
+      <c r="BL62" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM62" s="5">
+        <v>25</v>
+      </c>
+      <c r="BN62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO62" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP62" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ62" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR62" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="63" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B63">
+        <v>774</v>
+      </c>
+      <c r="C63" t="s">
+        <v>231</v>
+      </c>
+      <c r="D63">
+        <v>50</v>
+      </c>
+      <c r="E63" t="s">
+        <v>171</v>
+      </c>
+      <c r="F63">
+        <v>2</v>
+      </c>
+      <c r="G63">
+        <v>4880</v>
+      </c>
+      <c r="H63" t="s">
+        <v>21</v>
+      </c>
+      <c r="I63">
+        <v>74</v>
+      </c>
+      <c r="J63" t="s">
+        <v>22</v>
+      </c>
+      <c r="K63">
+        <v>14</v>
+      </c>
+      <c r="L63" t="s">
+        <v>135</v>
+      </c>
+      <c r="M63">
+        <v>65</v>
+      </c>
+      <c r="N63" t="s">
+        <v>171</v>
+      </c>
+      <c r="O63">
+        <v>1027</v>
+      </c>
+      <c r="P63" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q63">
+        <v>15</v>
+      </c>
+      <c r="R63" t="s">
+        <v>135</v>
+      </c>
+      <c r="S63">
+        <v>19</v>
+      </c>
+      <c r="T63" t="s">
+        <v>135</v>
+      </c>
+      <c r="U63">
+        <v>75</v>
+      </c>
+      <c r="V63" t="s">
+        <v>173</v>
+      </c>
+      <c r="W63">
+        <v>117.8</v>
+      </c>
+      <c r="X63" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y63">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="Z63" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA63">
+        <v>12.4</v>
+      </c>
+      <c r="AB63" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC63">
+        <v>44.4</v>
+      </c>
+      <c r="AD63" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE63">
+        <v>270</v>
+      </c>
+      <c r="AF63" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG63">
+        <v>320</v>
+      </c>
+      <c r="AH63" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI63">
+        <v>220</v>
+      </c>
+      <c r="AJ63" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK63">
+        <v>11.35</v>
+      </c>
+      <c r="AL63" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM63">
+        <v>1.18</v>
+      </c>
+      <c r="AN63" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO63" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP63" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ63">
+        <v>20</v>
+      </c>
+      <c r="AR63" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS63">
+        <v>861.24</v>
+      </c>
+      <c r="AT63" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU63">
+        <v>176.48</v>
+      </c>
+      <c r="AV63" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW63">
+        <v>116.5</v>
+      </c>
+      <c r="AX63" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY63">
+        <v>75.8</v>
+      </c>
+      <c r="AZ63" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA63" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB63" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC63">
+        <v>347.7</v>
+      </c>
+      <c r="BD63" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE63">
+        <v>241.7</v>
+      </c>
+      <c r="BF63" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG63" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH63" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI63">
+        <v>178.08</v>
+      </c>
+      <c r="BJ63" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK63">
+        <v>1000</v>
+      </c>
+      <c r="BL63" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM63">
+        <v>25</v>
+      </c>
+      <c r="BN63" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO63" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP63" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ63" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR63" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="64" spans="2:70" x14ac:dyDescent="0.3">
+      <c r="B64">
+        <v>774</v>
+      </c>
+      <c r="C64" t="s">
+        <v>231</v>
+      </c>
+      <c r="D64">
+        <v>75</v>
+      </c>
+      <c r="E64" t="s">
+        <v>171</v>
+      </c>
+      <c r="F64">
+        <v>3</v>
+      </c>
+      <c r="G64">
+        <v>7320</v>
+      </c>
+      <c r="H64" t="s">
+        <v>21</v>
+      </c>
+      <c r="I64">
+        <v>84</v>
+      </c>
+      <c r="J64" t="s">
+        <v>22</v>
+      </c>
+      <c r="K64">
+        <v>12</v>
+      </c>
+      <c r="L64" t="s">
+        <v>135</v>
+      </c>
+      <c r="M64">
+        <v>62</v>
+      </c>
+      <c r="N64" t="s">
+        <v>171</v>
+      </c>
+      <c r="O64">
+        <v>1027</v>
+      </c>
+      <c r="P64" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q64">
+        <v>15.7</v>
+      </c>
+      <c r="R64" t="s">
+        <v>135</v>
+      </c>
+      <c r="S64">
+        <v>22</v>
+      </c>
+      <c r="T64" t="s">
+        <v>135</v>
+      </c>
+      <c r="U64">
+        <v>140</v>
+      </c>
+      <c r="V64" t="s">
+        <v>173</v>
+      </c>
+      <c r="W64">
+        <v>140.6</v>
+      </c>
+      <c r="X64" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y64">
+        <v>102.6</v>
+      </c>
+      <c r="Z64" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA64">
+        <v>16.39</v>
+      </c>
+      <c r="AB64" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC64">
+        <v>57.4</v>
+      </c>
+      <c r="AD64" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE64">
+        <v>295</v>
+      </c>
+      <c r="AF64" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG64">
+        <v>355</v>
+      </c>
+      <c r="AH64" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI64">
+        <v>200</v>
+      </c>
+      <c r="AJ64" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK64">
+        <v>14.372</v>
+      </c>
+      <c r="AL64" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM64">
+        <v>2.23</v>
+      </c>
+      <c r="AN64" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO64" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP64" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ64">
+        <v>21</v>
+      </c>
+      <c r="AR64" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS64">
+        <v>1228.67</v>
+      </c>
+      <c r="AT64" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU64">
+        <v>172.76</v>
+      </c>
+      <c r="AV64" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW64">
+        <v>139.5</v>
+      </c>
+      <c r="AX64" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY64">
+        <v>101.2</v>
+      </c>
+      <c r="AZ64" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA64" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB64" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC64">
+        <v>381.8</v>
+      </c>
+      <c r="BD64" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE64">
+        <v>220.7</v>
+      </c>
+      <c r="BF64" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG64" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH64" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI64">
+        <v>169.05</v>
+      </c>
+      <c r="BJ64" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK64">
+        <v>1000</v>
+      </c>
+      <c r="BL64" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM64">
+        <v>25</v>
+      </c>
+      <c r="BN64" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO64" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP64" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ64" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR64" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="65" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="B65">
+        <v>774</v>
+      </c>
+      <c r="C65" t="s">
+        <v>231</v>
+      </c>
+      <c r="D65">
+        <v>85</v>
+      </c>
+      <c r="E65" t="s">
+        <v>171</v>
+      </c>
+      <c r="F65">
+        <v>4</v>
+      </c>
+      <c r="G65">
+        <v>8296</v>
+      </c>
+      <c r="H65" t="s">
+        <v>21</v>
+      </c>
+      <c r="I65">
+        <v>88</v>
+      </c>
+      <c r="J65" t="s">
+        <v>22</v>
+      </c>
+      <c r="K65">
+        <v>12</v>
+      </c>
+      <c r="L65" t="s">
+        <v>135</v>
+      </c>
+      <c r="M65">
+        <v>62</v>
+      </c>
+      <c r="N65" t="s">
+        <v>171</v>
+      </c>
+      <c r="O65">
+        <v>1027</v>
+      </c>
+      <c r="P65" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q65">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="R65" t="s">
+        <v>135</v>
+      </c>
+      <c r="S65">
+        <v>27</v>
+      </c>
+      <c r="T65" t="s">
+        <v>135</v>
+      </c>
+      <c r="U65">
+        <v>190</v>
+      </c>
+      <c r="V65" t="s">
+        <v>173</v>
+      </c>
+      <c r="W65">
+        <v>152.19999999999999</v>
+      </c>
+      <c r="X65" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y65">
+        <v>114.6</v>
+      </c>
+      <c r="Z65" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA65">
+        <v>17.73</v>
+      </c>
+      <c r="AB65" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC65">
+        <v>61</v>
+      </c>
+      <c r="AD65" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE65">
+        <v>310</v>
+      </c>
+      <c r="AF65" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG65">
+        <v>375</v>
+      </c>
+      <c r="AH65" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI65">
+        <v>205</v>
+      </c>
+      <c r="AJ65" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK65">
+        <v>15.108000000000001</v>
+      </c>
+      <c r="AL65" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM65">
+        <v>2.56</v>
+      </c>
+      <c r="AN65" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO65" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP65" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ65">
+        <v>22</v>
+      </c>
+      <c r="AR65" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS65">
+        <v>1422.92</v>
+      </c>
+      <c r="AT65" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU65">
+        <v>171.52</v>
+      </c>
+      <c r="AV65" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW65">
+        <v>152.19999999999999</v>
+      </c>
+      <c r="AX65" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY65">
+        <v>111</v>
+      </c>
+      <c r="AZ65" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA65" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB65" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC65">
+        <v>397.1</v>
+      </c>
+      <c r="BD65" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE65">
+        <v>220.9</v>
+      </c>
+      <c r="BF65" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG65" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH65" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI65">
+        <v>172.2</v>
+      </c>
+      <c r="BJ65" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK65">
+        <v>1000</v>
+      </c>
+      <c r="BL65" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM65">
+        <v>25</v>
+      </c>
+      <c r="BN65" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO65" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP65" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ65" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR65" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="66" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="B66">
+        <v>774</v>
+      </c>
+      <c r="C66" t="s">
+        <v>231</v>
+      </c>
+      <c r="D66">
+        <v>100</v>
+      </c>
+      <c r="E66" t="s">
+        <v>171</v>
+      </c>
+      <c r="F66">
+        <v>5</v>
+      </c>
+      <c r="G66">
+        <v>9760</v>
+      </c>
+      <c r="H66" t="s">
+        <v>21</v>
+      </c>
+      <c r="I66">
+        <v>93</v>
+      </c>
+      <c r="J66" t="s">
+        <v>22</v>
+      </c>
+      <c r="K66">
+        <v>12</v>
+      </c>
+      <c r="L66" t="s">
+        <v>135</v>
+      </c>
+      <c r="M66">
+        <v>62</v>
+      </c>
+      <c r="N66" t="s">
+        <v>171</v>
+      </c>
+      <c r="O66">
+        <v>1028</v>
+      </c>
+      <c r="P66" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q66">
+        <v>17</v>
+      </c>
+      <c r="R66" t="s">
+        <v>135</v>
+      </c>
+      <c r="S66">
+        <v>30</v>
+      </c>
+      <c r="T66" t="s">
+        <v>135</v>
+      </c>
+      <c r="U66">
+        <v>250</v>
+      </c>
+      <c r="V66" t="s">
+        <v>173</v>
+      </c>
+      <c r="W66">
+        <v>147.6</v>
+      </c>
+      <c r="X66" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y66">
+        <v>129.6</v>
+      </c>
+      <c r="Z66" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA66">
+        <v>19.739999999999998</v>
+      </c>
+      <c r="AB66" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC66">
+        <v>70.5</v>
+      </c>
+      <c r="AD66" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE66">
+        <v>362</v>
+      </c>
+      <c r="AF66" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG66">
+        <v>425</v>
+      </c>
+      <c r="AH66" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI66">
+        <v>230</v>
+      </c>
+      <c r="AJ66" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK66">
+        <v>16.654</v>
+      </c>
+      <c r="AL66" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM66">
+        <v>3.28</v>
+      </c>
+      <c r="AN66" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO66" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP66" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ66">
+        <v>24</v>
+      </c>
+      <c r="AR66" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS66">
+        <v>1690.14</v>
+      </c>
+      <c r="AT66" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU66">
+        <v>173.17</v>
+      </c>
+      <c r="AV66" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW66">
+        <v>147.6</v>
+      </c>
+      <c r="AX66" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY66">
+        <v>126.2</v>
+      </c>
+      <c r="AZ66" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA66" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB66" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC66">
+        <v>446.8</v>
+      </c>
+      <c r="BD66" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE66">
+        <v>245.6</v>
+      </c>
+      <c r="BF66" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG66" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH66" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI66">
+        <v>173.54</v>
+      </c>
+      <c r="BJ66" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK66">
+        <v>1000</v>
+      </c>
+      <c r="BL66" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM66">
+        <v>25</v>
+      </c>
+      <c r="BN66" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO66" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP66" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ66" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR66" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="67" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="B67">
+        <v>774</v>
+      </c>
+      <c r="C67" t="s">
+        <v>231</v>
+      </c>
+      <c r="D67">
+        <v>110</v>
+      </c>
+      <c r="E67" t="s">
+        <v>171</v>
+      </c>
+      <c r="F67">
+        <v>6</v>
+      </c>
+      <c r="G67">
+        <v>10736</v>
+      </c>
+      <c r="H67" t="s">
+        <v>21</v>
+      </c>
+      <c r="I67">
+        <v>96</v>
+      </c>
+      <c r="J67" t="s">
+        <v>22</v>
+      </c>
+      <c r="K67">
+        <v>13</v>
+      </c>
+      <c r="L67" t="s">
+        <v>135</v>
+      </c>
+      <c r="M67">
+        <v>62</v>
+      </c>
+      <c r="N67" t="s">
+        <v>171</v>
+      </c>
+      <c r="O67">
+        <v>1027</v>
+      </c>
+      <c r="P67" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q67">
+        <v>18</v>
+      </c>
+      <c r="R67" t="s">
+        <v>135</v>
+      </c>
+      <c r="S67">
+        <v>28</v>
+      </c>
+      <c r="T67" t="s">
+        <v>135</v>
+      </c>
+      <c r="U67">
+        <v>285</v>
+      </c>
+      <c r="V67" t="s">
+        <v>173</v>
+      </c>
+      <c r="W67">
+        <v>153.6</v>
+      </c>
+      <c r="X67" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y67">
+        <v>142.80000000000001</v>
+      </c>
+      <c r="Z67" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA67">
+        <v>21.03</v>
+      </c>
+      <c r="AB67" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC67">
+        <v>75.3</v>
+      </c>
+      <c r="AD67" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE67">
+        <v>389</v>
+      </c>
+      <c r="AF67" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG67">
+        <v>450</v>
+      </c>
+      <c r="AH67" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI67">
+        <v>245</v>
+      </c>
+      <c r="AJ67" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK67">
+        <v>17.189</v>
+      </c>
+      <c r="AL67" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM67">
+        <v>3.45</v>
+      </c>
+      <c r="AN67" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO67" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP67" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ67">
+        <v>24</v>
+      </c>
+      <c r="AR67" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS67">
+        <v>1935.48</v>
+      </c>
+      <c r="AT67" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU67">
+        <v>180.28</v>
+      </c>
+      <c r="AV67" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW67">
+        <v>153.6</v>
+      </c>
+      <c r="AX67" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY67">
+        <v>140.80000000000001</v>
+      </c>
+      <c r="AZ67" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA67" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB67" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC67">
+        <v>473.9</v>
+      </c>
+      <c r="BD67" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE67">
+        <v>261</v>
+      </c>
+      <c r="BF67" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG67" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH67" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI67">
+        <v>180.84</v>
+      </c>
+      <c r="BJ67" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK67">
+        <v>1000</v>
+      </c>
+      <c r="BL67" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM67">
+        <v>25</v>
+      </c>
+      <c r="BN67" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO67" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP67" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ67" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR67" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="68" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="B68">
+        <v>774</v>
+      </c>
+      <c r="C68" t="s">
+        <v>231</v>
+      </c>
+      <c r="D68">
+        <v>100</v>
+      </c>
+      <c r="E68" t="s">
+        <v>171</v>
+      </c>
+      <c r="F68">
+        <v>7</v>
+      </c>
+      <c r="G68">
+        <v>9760</v>
+      </c>
+      <c r="H68" t="s">
+        <v>21</v>
+      </c>
+      <c r="I68">
+        <v>93</v>
+      </c>
+      <c r="J68" t="s">
+        <v>22</v>
+      </c>
+      <c r="K68">
+        <v>12</v>
+      </c>
+      <c r="L68" t="s">
+        <v>135</v>
+      </c>
+      <c r="M68">
+        <v>62</v>
+      </c>
+      <c r="N68" t="s">
+        <v>171</v>
+      </c>
+      <c r="O68">
+        <v>1028</v>
+      </c>
+      <c r="P68" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q68">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="R68" t="s">
+        <v>135</v>
+      </c>
+      <c r="S68">
+        <v>30</v>
+      </c>
+      <c r="T68" t="s">
+        <v>135</v>
+      </c>
+      <c r="U68">
+        <v>250</v>
+      </c>
+      <c r="V68" t="s">
+        <v>173</v>
+      </c>
+      <c r="W68">
+        <v>147.80000000000001</v>
+      </c>
+      <c r="X68" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y68">
+        <v>134</v>
+      </c>
+      <c r="Z68" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA68">
+        <v>19.739999999999998</v>
+      </c>
+      <c r="AB68" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC68">
+        <v>71</v>
+      </c>
+      <c r="AD68" t="s">
+        <v>171</v>
+      </c>
+      <c r="AE68">
+        <v>364</v>
+      </c>
+      <c r="AF68" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG68">
+        <v>425</v>
+      </c>
+      <c r="AH68" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI68">
+        <v>230</v>
+      </c>
+      <c r="AJ68" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK68">
+        <v>16.622</v>
+      </c>
+      <c r="AL68" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM68">
+        <v>3.26</v>
+      </c>
+      <c r="AN68" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO68" t="s">
+        <v>231</v>
+      </c>
+      <c r="AP68" t="s">
+        <v>224</v>
+      </c>
+      <c r="AQ68">
+        <v>23</v>
+      </c>
+      <c r="AR68" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS68">
+        <v>1698.11</v>
+      </c>
+      <c r="AT68" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU68">
+        <v>173.99</v>
+      </c>
+      <c r="AV68" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW68">
+        <v>147.80000000000001</v>
+      </c>
+      <c r="AX68" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY68">
+        <v>130.80000000000001</v>
+      </c>
+      <c r="AZ68" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA68" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB68" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC68">
+        <v>446.3</v>
+      </c>
+      <c r="BD68" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE68">
+        <v>245.1</v>
+      </c>
+      <c r="BF68" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG68" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH68" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI68">
+        <v>174.34</v>
+      </c>
+      <c r="BJ68" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK68">
+        <v>1000</v>
+      </c>
+      <c r="BL68" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM68">
+        <v>25</v>
+      </c>
+      <c r="BN68" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO68" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP68" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ68" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR68" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="69" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>231</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C69" t="s">
+        <v>231</v>
+      </c>
+      <c r="D69">
+        <v>50</v>
+      </c>
+      <c r="E69" t="s">
+        <v>171</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+      <c r="G69" s="4">
+        <v>3135</v>
+      </c>
+      <c r="H69" t="s">
+        <v>21</v>
+      </c>
+      <c r="I69">
+        <v>114</v>
+      </c>
+      <c r="J69" t="s">
+        <v>22</v>
+      </c>
+      <c r="K69">
+        <v>15</v>
+      </c>
+      <c r="L69" t="s">
+        <v>135</v>
+      </c>
+      <c r="M69" t="s">
+        <v>231</v>
+      </c>
+      <c r="N69" t="s">
+        <v>171</v>
+      </c>
+      <c r="O69" t="s">
+        <v>231</v>
+      </c>
+      <c r="P69" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>231</v>
+      </c>
+      <c r="R69" t="s">
+        <v>135</v>
+      </c>
+      <c r="S69">
+        <v>34</v>
+      </c>
+      <c r="T69" t="s">
+        <v>135</v>
+      </c>
+      <c r="U69">
+        <v>80</v>
+      </c>
+      <c r="V69" t="s">
+        <v>173</v>
+      </c>
+      <c r="W69" t="s">
+        <v>231</v>
+      </c>
+      <c r="X69" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y69" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z69" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA69" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB69" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC69">
+        <v>43</v>
+      </c>
+      <c r="AD69" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE69">
+        <v>286</v>
+      </c>
+      <c r="AF69" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG69">
+        <v>340</v>
+      </c>
+      <c r="AH69" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI69">
+        <v>250</v>
+      </c>
+      <c r="AJ69" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK69">
+        <v>11.6</v>
+      </c>
+      <c r="AL69" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM69">
+        <v>1</v>
+      </c>
+      <c r="AN69" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO69">
+        <v>0.9</v>
+      </c>
+      <c r="AP69" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ69">
+        <v>130</v>
+      </c>
+      <c r="AR69" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS69" t="s">
+        <v>231</v>
+      </c>
+      <c r="AT69" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU69" t="s">
+        <v>231</v>
+      </c>
+      <c r="AV69" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW69" t="s">
+        <v>231</v>
+      </c>
+      <c r="AX69" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY69" t="s">
+        <v>231</v>
+      </c>
+      <c r="AZ69" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB69" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD69" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BF69" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH69" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BJ69" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BL69" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BN69" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP69" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR69" t="s">
+        <v>173</v>
+      </c>
+      <c r="BS69" t="s">
+        <v>231</v>
+      </c>
+      <c r="BT69" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="70" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>231</v>
+      </c>
+      <c r="B70" t="s">
+        <v>231</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D70">
+        <v>75</v>
+      </c>
+      <c r="E70" t="s">
+        <v>171</v>
+      </c>
+      <c r="F70">
+        <v>2</v>
+      </c>
+      <c r="G70">
+        <v>4927.5</v>
+      </c>
+      <c r="H70" t="s">
+        <v>21</v>
+      </c>
+      <c r="I70" s="4">
+        <v>120</v>
+      </c>
+      <c r="J70" t="s">
+        <v>22</v>
+      </c>
+      <c r="K70">
+        <v>15</v>
+      </c>
+      <c r="L70" t="s">
+        <v>135</v>
+      </c>
+      <c r="M70" t="s">
+        <v>231</v>
+      </c>
+      <c r="N70" t="s">
+        <v>171</v>
+      </c>
+      <c r="O70" t="s">
+        <v>231</v>
+      </c>
+      <c r="P70" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>231</v>
+      </c>
+      <c r="R70" t="s">
+        <v>135</v>
+      </c>
+      <c r="S70">
+        <v>39</v>
+      </c>
+      <c r="T70" t="s">
+        <v>135</v>
+      </c>
+      <c r="U70">
+        <v>180</v>
+      </c>
+      <c r="V70" t="s">
+        <v>173</v>
+      </c>
+      <c r="W70" t="s">
+        <v>231</v>
+      </c>
+      <c r="X70" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y70" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z70" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA70" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB70" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC70">
+        <v>54.8</v>
+      </c>
+      <c r="AD70" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE70">
+        <v>300</v>
+      </c>
+      <c r="AF70" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG70">
+        <v>360</v>
+      </c>
+      <c r="AH70" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI70">
+        <v>238</v>
+      </c>
+      <c r="AJ70" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK70">
+        <v>14.8</v>
+      </c>
+      <c r="AL70" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM70">
+        <v>1.8</v>
+      </c>
+      <c r="AN70" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO70">
+        <v>1.6</v>
+      </c>
+      <c r="AP70" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ70">
+        <v>130</v>
+      </c>
+      <c r="AR70" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS70" t="s">
+        <v>231</v>
+      </c>
+      <c r="AT70" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU70" t="s">
+        <v>231</v>
+      </c>
+      <c r="AV70" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW70" t="s">
+        <v>231</v>
+      </c>
+      <c r="AX70" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY70" t="s">
+        <v>231</v>
+      </c>
+      <c r="AZ70" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB70" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD70" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BF70" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH70" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BJ70" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BL70" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BN70" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP70" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR70" t="s">
+        <v>173</v>
+      </c>
+      <c r="BS70" t="s">
+        <v>231</v>
+      </c>
+      <c r="BT70" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="71" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>231</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C71" t="s">
+        <v>231</v>
+      </c>
+      <c r="D71">
+        <v>85</v>
+      </c>
+      <c r="E71" t="s">
+        <v>171</v>
+      </c>
+      <c r="F71">
+        <v>3</v>
+      </c>
+      <c r="G71" s="4">
+        <v>5548.3</v>
+      </c>
+      <c r="H71" t="s">
+        <v>21</v>
+      </c>
+      <c r="I71">
+        <v>122</v>
+      </c>
+      <c r="J71" t="s">
+        <v>22</v>
+      </c>
+      <c r="K71">
+        <v>15</v>
+      </c>
+      <c r="L71" t="s">
+        <v>135</v>
+      </c>
+      <c r="M71" t="s">
+        <v>231</v>
+      </c>
+      <c r="N71" t="s">
+        <v>171</v>
+      </c>
+      <c r="O71" t="s">
+        <v>231</v>
+      </c>
+      <c r="P71" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>231</v>
+      </c>
+      <c r="R71" t="s">
+        <v>135</v>
+      </c>
+      <c r="S71">
+        <v>40</v>
+      </c>
+      <c r="T71" t="s">
+        <v>135</v>
+      </c>
+      <c r="U71">
+        <v>210</v>
+      </c>
+      <c r="V71" t="s">
+        <v>173</v>
+      </c>
+      <c r="W71" t="s">
+        <v>231</v>
+      </c>
+      <c r="X71" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y71" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z71" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA71" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB71" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC71">
+        <v>60.6</v>
+      </c>
+      <c r="AD71" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE71">
+        <v>301</v>
+      </c>
+      <c r="AF71" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG71">
+        <v>365</v>
+      </c>
+      <c r="AH71" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI71">
+        <v>238</v>
+      </c>
+      <c r="AJ71" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK71">
+        <v>15.4</v>
+      </c>
+      <c r="AL71" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM71">
+        <v>2</v>
+      </c>
+      <c r="AN71" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO71">
+        <v>1.8</v>
+      </c>
+      <c r="AP71" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ71">
+        <v>130</v>
+      </c>
+      <c r="AR71" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS71" t="s">
+        <v>231</v>
+      </c>
+      <c r="AT71" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU71" t="s">
+        <v>231</v>
+      </c>
+      <c r="AV71" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW71" t="s">
+        <v>231</v>
+      </c>
+      <c r="AX71" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY71" t="s">
+        <v>231</v>
+      </c>
+      <c r="AZ71" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB71" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD71" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BF71" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH71" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BJ71" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BL71" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BN71" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP71" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR71" t="s">
+        <v>173</v>
+      </c>
+      <c r="BS71" t="s">
+        <v>231</v>
+      </c>
+      <c r="BT71" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="72" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>231</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C72" t="s">
+        <v>231</v>
+      </c>
+      <c r="D72">
+        <v>100</v>
+      </c>
+      <c r="E72" t="s">
+        <v>171</v>
+      </c>
+      <c r="F72">
+        <v>4</v>
+      </c>
+      <c r="G72" s="4">
+        <v>6580</v>
+      </c>
+      <c r="H72" t="s">
+        <v>21</v>
+      </c>
+      <c r="I72">
+        <v>127</v>
+      </c>
+      <c r="J72" t="s">
+        <v>22</v>
+      </c>
+      <c r="K72">
+        <v>15</v>
+      </c>
+      <c r="L72" t="s">
+        <v>135</v>
+      </c>
+      <c r="M72" t="s">
+        <v>231</v>
+      </c>
+      <c r="N72" t="s">
+        <v>171</v>
+      </c>
+      <c r="O72" t="s">
+        <v>231</v>
+      </c>
+      <c r="P72" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>231</v>
+      </c>
+      <c r="R72" t="s">
+        <v>135</v>
+      </c>
+      <c r="S72">
+        <v>43</v>
+      </c>
+      <c r="T72" t="s">
+        <v>135</v>
+      </c>
+      <c r="U72">
+        <v>265</v>
+      </c>
+      <c r="V72" t="s">
+        <v>173</v>
+      </c>
+      <c r="W72" t="s">
+        <v>231</v>
+      </c>
+      <c r="X72" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y72" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z72" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA72" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB72" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC72">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="AD72" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE72">
+        <v>335.6</v>
+      </c>
+      <c r="AF72" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG72">
+        <v>400</v>
+      </c>
+      <c r="AH72" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI72">
+        <v>245</v>
+      </c>
+      <c r="AJ72" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK72">
+        <v>17.010000000000002</v>
+      </c>
+      <c r="AL72" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM72">
+        <v>2.5</v>
+      </c>
+      <c r="AN72" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO72">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AP72" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ72">
+        <v>129</v>
+      </c>
+      <c r="AR72" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS72" t="s">
+        <v>231</v>
+      </c>
+      <c r="AT72" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU72" t="s">
+        <v>231</v>
+      </c>
+      <c r="AV72" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW72" t="s">
+        <v>231</v>
+      </c>
+      <c r="AX72" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY72" t="s">
+        <v>231</v>
+      </c>
+      <c r="AZ72" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB72" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD72" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BF72" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH72" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BJ72" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BL72" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BN72" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP72" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR72" t="s">
+        <v>173</v>
+      </c>
+      <c r="BS72" t="s">
+        <v>231</v>
+      </c>
+      <c r="BT72" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="73" spans="1:72" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>231</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C73" t="s">
+        <v>231</v>
+      </c>
+      <c r="D73">
+        <v>110</v>
+      </c>
+      <c r="E73" t="s">
+        <v>171</v>
+      </c>
+      <c r="F73">
+        <v>5</v>
+      </c>
+      <c r="G73">
+        <v>7240</v>
+      </c>
+      <c r="H73" t="s">
+        <v>21</v>
+      </c>
+      <c r="I73">
+        <v>130</v>
+      </c>
+      <c r="J73" t="s">
+        <v>22</v>
+      </c>
+      <c r="K73">
+        <v>15</v>
+      </c>
+      <c r="L73" t="s">
+        <v>135</v>
+      </c>
+      <c r="M73" t="s">
+        <v>231</v>
+      </c>
+      <c r="N73" t="s">
+        <v>171</v>
+      </c>
+      <c r="O73" t="s">
+        <v>231</v>
+      </c>
+      <c r="P73" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>231</v>
+      </c>
+      <c r="R73" t="s">
+        <v>135</v>
+      </c>
+      <c r="S73">
+        <v>46</v>
+      </c>
+      <c r="T73" t="s">
+        <v>135</v>
+      </c>
+      <c r="U73">
+        <v>260</v>
+      </c>
+      <c r="V73" t="s">
+        <v>173</v>
+      </c>
+      <c r="W73" t="s">
+        <v>231</v>
+      </c>
+      <c r="X73" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y73" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z73" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA73" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB73" t="s">
+        <v>174</v>
+      </c>
+      <c r="AC73">
+        <v>76.2</v>
+      </c>
+      <c r="AD73" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE73">
+        <v>342</v>
+      </c>
+      <c r="AF73" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG73">
+        <v>420</v>
+      </c>
+      <c r="AH73" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI73">
+        <v>250</v>
+      </c>
+      <c r="AJ73" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK73">
+        <v>17.5</v>
+      </c>
+      <c r="AL73" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM73">
+        <v>2.8</v>
+      </c>
+      <c r="AN73" t="s">
+        <v>174</v>
+      </c>
+      <c r="AO73">
+        <v>2.6</v>
+      </c>
+      <c r="AP73" t="s">
+        <v>174</v>
+      </c>
+      <c r="AQ73">
+        <v>130</v>
+      </c>
+      <c r="AR73" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS73" t="s">
+        <v>231</v>
+      </c>
+      <c r="AT73" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU73" t="s">
+        <v>231</v>
+      </c>
+      <c r="AV73" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW73" t="s">
+        <v>231</v>
+      </c>
+      <c r="AX73" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY73" t="s">
+        <v>231</v>
+      </c>
+      <c r="AZ73" t="s">
+        <v>174</v>
+      </c>
+      <c r="BA73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BB73" t="s">
+        <v>224</v>
+      </c>
+      <c r="BC73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD73" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BF73" t="s">
+        <v>135</v>
+      </c>
+      <c r="BG73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BH73" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BJ73" t="s">
+        <v>20</v>
+      </c>
+      <c r="BK73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BL73" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BN73" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BP73" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BR73" t="s">
+        <v>173</v>
+      </c>
+      <c r="BS73" t="s">
+        <v>231</v>
+      </c>
+      <c r="BT73" t="s">
+        <v>231</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
name changes in excel
</commit_message>
<xml_diff>
--- a/Aepms-backend/data/Engine_Performance_Data.xlsx
+++ b/Aepms-backend/data/Engine_Performance_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GOKUL\Desktop\WORKPLACE\Workplace\Aepms-backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656CD45D-1287-449F-BEAF-3CE83B132A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACAD501-58C8-4E4D-ABA2-BDBB79A7EC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vessel_info" sheetId="1" r:id="rId1"/>
@@ -574,9 +574,6 @@
     <t>kg/h</t>
   </si>
   <si>
-    <t>GCL Narmadha</t>
-  </si>
-  <si>
     <t>Summary Data of Shop Trial</t>
   </si>
   <si>
@@ -815,6 +812,9 @@
   </si>
   <si>
     <t>DAIHATSU DIESEL MFG. CO., LTD.</t>
+  </si>
+  <si>
+    <t>GCL Narmada</t>
   </si>
 </sst>
 </file>
@@ -1544,25 +1544,25 @@
         <v>127</v>
       </c>
       <c r="T1" t="s">
+        <v>201</v>
+      </c>
+      <c r="U1" t="s">
         <v>202</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>203</v>
       </c>
-      <c r="V1" t="s">
-        <v>204</v>
-      </c>
       <c r="W1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="X1" t="s">
+        <v>214</v>
+      </c>
+      <c r="Y1" t="s">
         <v>215</v>
       </c>
-      <c r="Y1" t="s">
-        <v>216</v>
-      </c>
       <c r="Z1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AA1" t="s">
         <v>11</v>
@@ -1647,13 +1647,13 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>178</v>
+        <v>258</v>
       </c>
       <c r="C3">
         <v>9481685</v>
       </c>
       <c r="D3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E3" t="s">
         <v>15</v>
@@ -1721,16 +1721,16 @@
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C4">
         <v>9481661</v>
       </c>
       <c r="D4" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" t="s">
         <v>182</v>
-      </c>
-      <c r="E4" t="s">
-        <v>183</v>
       </c>
       <c r="F4" t="s">
         <v>16</v>
@@ -1739,7 +1739,7 @@
         <v>17</v>
       </c>
       <c r="H4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I4" t="s">
         <v>123</v>
@@ -1795,16 +1795,16 @@
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C5">
         <v>9481659</v>
       </c>
       <c r="D5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F5" t="s">
         <v>16</v>
@@ -1813,7 +1813,7 @@
         <v>17</v>
       </c>
       <c r="H5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I5" t="s">
         <v>123</v>
@@ -1869,16 +1869,16 @@
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C6">
         <v>9481219</v>
       </c>
       <c r="D6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F6" t="s">
         <v>16</v>
@@ -1887,7 +1887,7 @@
         <v>17</v>
       </c>
       <c r="H6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I6" t="s">
         <v>123</v>
@@ -1943,31 +1943,31 @@
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C7">
         <v>9832913</v>
       </c>
       <c r="D7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F7" t="s">
         <v>190</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>191</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>192</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>193</v>
       </c>
-      <c r="I7" t="s">
-        <v>194</v>
-      </c>
       <c r="J7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K7">
         <v>6</v>
@@ -2017,31 +2017,31 @@
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C8">
         <v>9832925</v>
       </c>
       <c r="D8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E8" t="s">
+        <v>189</v>
+      </c>
+      <c r="F8" t="s">
         <v>190</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>191</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>192</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>193</v>
       </c>
-      <c r="I8" t="s">
-        <v>194</v>
-      </c>
       <c r="J8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K8">
         <v>6</v>
@@ -2091,31 +2091,31 @@
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C9">
         <v>9792058</v>
       </c>
       <c r="D9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E9" s="2">
         <v>1576</v>
       </c>
       <c r="F9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G9" t="s">
+        <v>208</v>
+      </c>
+      <c r="H9" t="s">
         <v>209</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>210</v>
       </c>
-      <c r="I9" t="s">
-        <v>211</v>
-      </c>
       <c r="J9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K9">
         <v>6</v>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C10">
         <v>9532082</v>
@@ -2168,22 +2168,22 @@
         <v>5933</v>
       </c>
       <c r="E10" t="s">
+        <v>244</v>
+      </c>
+      <c r="F10" t="s">
+        <v>233</v>
+      </c>
+      <c r="G10" t="s">
         <v>245</v>
       </c>
-      <c r="F10" t="s">
-        <v>234</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
+        <v>232</v>
+      </c>
+      <c r="I10" t="s">
+        <v>231</v>
+      </c>
+      <c r="J10" t="s">
         <v>246</v>
-      </c>
-      <c r="H10" t="s">
-        <v>233</v>
-      </c>
-      <c r="I10" t="s">
-        <v>232</v>
-      </c>
-      <c r="J10" t="s">
-        <v>247</v>
       </c>
       <c r="K10">
         <v>6</v>
@@ -2221,31 +2221,31 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C11">
         <v>9521813</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F11" t="s">
         <v>220</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>221</v>
       </c>
-      <c r="G11" t="s">
-        <v>222</v>
-      </c>
       <c r="H11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K11">
         <v>5</v>
@@ -2286,7 +2286,7 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C12">
         <v>9628893</v>
@@ -2295,22 +2295,22 @@
         <v>774</v>
       </c>
       <c r="E12" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F12" t="s">
+        <v>248</v>
+      </c>
+      <c r="G12" t="s">
         <v>249</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>250</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
+        <v>238</v>
+      </c>
+      <c r="J12" t="s">
         <v>251</v>
-      </c>
-      <c r="I12" t="s">
-        <v>239</v>
-      </c>
-      <c r="J12" t="s">
-        <v>252</v>
       </c>
       <c r="K12">
         <v>5</v>
@@ -2348,7 +2348,7 @@
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C13">
         <v>9644500</v>
@@ -2360,19 +2360,19 @@
         <v>10701</v>
       </c>
       <c r="F13" t="s">
+        <v>224</v>
+      </c>
+      <c r="G13" t="s">
         <v>225</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>226</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>227</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>228</v>
-      </c>
-      <c r="J13" t="s">
-        <v>229</v>
       </c>
       <c r="K13">
         <v>6</v>
@@ -2410,31 +2410,31 @@
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C14">
         <v>9628910</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E14" t="s">
+        <v>235</v>
+      </c>
+      <c r="F14" t="s">
+        <v>237</v>
+      </c>
+      <c r="G14" t="s">
         <v>236</v>
       </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
+        <v>239</v>
+      </c>
+      <c r="I14" t="s">
         <v>238</v>
       </c>
-      <c r="G14" t="s">
-        <v>237</v>
-      </c>
-      <c r="H14" t="s">
-        <v>240</v>
-      </c>
-      <c r="I14" t="s">
-        <v>239</v>
-      </c>
       <c r="J14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="K14">
         <v>5</v>
@@ -2461,22 +2461,22 @@
         <v>22</v>
       </c>
       <c r="T14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="U14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="W14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="X14" t="s">
         <v>21</v>
       </c>
       <c r="Y14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z14" t="s">
         <v>171</v>
@@ -2484,31 +2484,31 @@
     </row>
     <row r="15" spans="1:28" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C15">
         <v>9486295</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="F15" t="s">
         <v>254</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>255</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="I15" t="s">
         <v>256</v>
       </c>
-      <c r="H15" s="16" t="s">
-        <v>258</v>
-      </c>
-      <c r="I15" t="s">
-        <v>257</v>
-      </c>
       <c r="J15" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="K15">
         <v>8</v>
@@ -2544,13 +2544,13 @@
         <v>73</v>
       </c>
       <c r="W15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="X15" t="s">
         <v>21</v>
       </c>
       <c r="Y15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z15" t="s">
         <v>171</v>
@@ -2685,7 +2685,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C3" s="1">
         <v>40518</v>
@@ -2697,7 +2697,7 @@
         <v>132</v>
       </c>
       <c r="F3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G3" t="s">
         <v>134</v>
@@ -2726,7 +2726,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C4" s="1">
         <v>40518</v>
@@ -2738,7 +2738,7 @@
         <v>132</v>
       </c>
       <c r="F4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G4" t="s">
         <v>134</v>
@@ -2767,7 +2767,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C5" s="1">
         <v>40518</v>
@@ -2779,7 +2779,7 @@
         <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G5" t="s">
         <v>134</v>
@@ -2808,7 +2808,7 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C6" s="1">
         <v>40518</v>
@@ -2820,7 +2820,7 @@
         <v>132</v>
       </c>
       <c r="F6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G6" t="s">
         <v>134</v>
@@ -2849,7 +2849,7 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C7" s="1">
         <v>43461</v>
@@ -2858,13 +2858,13 @@
         <v>131</v>
       </c>
       <c r="E7" t="s">
+        <v>194</v>
+      </c>
+      <c r="F7" t="s">
         <v>195</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>196</v>
-      </c>
-      <c r="G7" t="s">
-        <v>197</v>
       </c>
       <c r="H7">
         <v>6</v>
@@ -2893,7 +2893,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C8" s="1">
         <v>43461</v>
@@ -2902,13 +2902,13 @@
         <v>131</v>
       </c>
       <c r="E8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H8">
         <v>6</v>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C9" s="1">
         <v>42788</v>
@@ -2946,13 +2946,13 @@
         <v>131</v>
       </c>
       <c r="E9" t="s">
+        <v>205</v>
+      </c>
+      <c r="F9" t="s">
         <v>206</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>207</v>
-      </c>
-      <c r="G9" t="s">
-        <v>208</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -3001,7 +3001,7 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C11" s="1">
         <v>42788</v>
@@ -3079,7 +3079,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C14" s="1">
         <v>42788</v>
@@ -3105,7 +3105,7 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C15" s="1">
         <v>42788</v>
@@ -4877,7 +4877,7 @@
     </row>
     <row r="9" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D9">
         <v>25</v>
@@ -5083,7 +5083,7 @@
     </row>
     <row r="10" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D10">
         <v>50</v>
@@ -5289,7 +5289,7 @@
     </row>
     <row r="11" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D11">
         <v>75</v>
@@ -5495,7 +5495,7 @@
     </row>
     <row r="12" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D12">
         <v>90</v>
@@ -5701,7 +5701,7 @@
     </row>
     <row r="13" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D13">
         <v>100</v>
@@ -5907,7 +5907,7 @@
     </row>
     <row r="14" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D14">
         <v>100</v>
@@ -6113,7 +6113,7 @@
     </row>
     <row r="15" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D15">
         <v>110</v>
@@ -6319,7 +6319,7 @@
     </row>
     <row r="16" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D16">
         <v>25</v>
@@ -6525,7 +6525,7 @@
     </row>
     <row r="17" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D17">
         <v>50</v>
@@ -6731,7 +6731,7 @@
     </row>
     <row r="18" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D18">
         <v>75</v>
@@ -6937,7 +6937,7 @@
     </row>
     <row r="19" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D19">
         <v>90</v>
@@ -7143,7 +7143,7 @@
     </row>
     <row r="20" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D20">
         <v>100</v>
@@ -7349,7 +7349,7 @@
     </row>
     <row r="21" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D21">
         <v>100</v>
@@ -7555,7 +7555,7 @@
     </row>
     <row r="22" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D22">
         <v>110</v>
@@ -7761,7 +7761,7 @@
     </row>
     <row r="23" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D23">
         <v>25</v>
@@ -7967,7 +7967,7 @@
     </row>
     <row r="24" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -8173,7 +8173,7 @@
     </row>
     <row r="25" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D25">
         <v>75</v>
@@ -8379,7 +8379,7 @@
     </row>
     <row r="26" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D26">
         <v>90</v>
@@ -8585,7 +8585,7 @@
     </row>
     <row r="27" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D27">
         <v>100</v>
@@ -8791,7 +8791,7 @@
     </row>
     <row r="28" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D28">
         <v>100</v>
@@ -8997,7 +8997,7 @@
     </row>
     <row r="29" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D29">
         <v>110</v>
@@ -9203,7 +9203,7 @@
     </row>
     <row r="30" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D30">
         <v>25</v>
@@ -9409,7 +9409,7 @@
     </row>
     <row r="31" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D31">
         <v>50</v>
@@ -9615,7 +9615,7 @@
     </row>
     <row r="32" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D32">
         <v>75</v>
@@ -9821,7 +9821,7 @@
     </row>
     <row r="33" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D33">
         <v>90</v>
@@ -10027,7 +10027,7 @@
     </row>
     <row r="34" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D34">
         <v>100</v>
@@ -10233,7 +10233,7 @@
     </row>
     <row r="35" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D35">
         <v>100</v>
@@ -10439,7 +10439,7 @@
     </row>
     <row r="36" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D36">
         <v>110</v>
@@ -10645,7 +10645,7 @@
     </row>
     <row r="37" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D37">
         <v>25</v>
@@ -10845,7 +10845,7 @@
     </row>
     <row r="38" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D38">
         <v>50</v>
@@ -11045,7 +11045,7 @@
     </row>
     <row r="39" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D39">
         <v>75</v>
@@ -11245,7 +11245,7 @@
     </row>
     <row r="40" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D40">
         <v>100</v>
@@ -11445,7 +11445,7 @@
     </row>
     <row r="41" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D41">
         <v>100</v>
@@ -11645,7 +11645,7 @@
     </row>
     <row r="42" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D42">
         <v>110</v>
@@ -11845,7 +11845,7 @@
     </row>
     <row r="43" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D43">
         <v>25</v>
@@ -12045,7 +12045,7 @@
     </row>
     <row r="44" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D44">
         <v>50</v>
@@ -12245,7 +12245,7 @@
     </row>
     <row r="45" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D45">
         <v>75</v>
@@ -12445,7 +12445,7 @@
     </row>
     <row r="46" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D46">
         <v>100</v>
@@ -12645,7 +12645,7 @@
     </row>
     <row r="47" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D47">
         <v>100</v>
@@ -12845,7 +12845,7 @@
     </row>
     <row r="48" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D48">
         <v>110</v>
@@ -13045,7 +13045,7 @@
     </row>
     <row r="49" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D49">
         <v>25</v>
@@ -13159,7 +13159,7 @@
         <v>0.38</v>
       </c>
       <c r="AP49" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ49">
         <v>33</v>
@@ -13195,7 +13195,7 @@
         <v>0.43</v>
       </c>
       <c r="BB49" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC49">
         <v>217</v>
@@ -13245,7 +13245,7 @@
     </row>
     <row r="50" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D50">
         <v>50</v>
@@ -13359,7 +13359,7 @@
         <v>1.06</v>
       </c>
       <c r="AP50" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ50">
         <v>32</v>
@@ -13395,7 +13395,7 @@
         <v>1.0900000000000001</v>
       </c>
       <c r="BB50" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC50">
         <v>311</v>
@@ -13445,7 +13445,7 @@
     </row>
     <row r="51" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D51">
         <v>65</v>
@@ -13559,7 +13559,7 @@
         <v>1.66</v>
       </c>
       <c r="AP51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ51">
         <v>33</v>
@@ -13595,7 +13595,7 @@
         <v>1.68</v>
       </c>
       <c r="BB51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC51">
         <v>329</v>
@@ -13645,7 +13645,7 @@
     </row>
     <row r="52" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D52">
         <v>75.599999999999994</v>
@@ -13759,7 +13759,7 @@
         <v>2.06</v>
       </c>
       <c r="AP52" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ52">
         <v>32</v>
@@ -13795,7 +13795,7 @@
         <v>2.0699999999999998</v>
       </c>
       <c r="BB52" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC52">
         <v>349</v>
@@ -13845,7 +13845,7 @@
     </row>
     <row r="53" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D53">
         <v>85</v>
@@ -13959,7 +13959,7 @@
         <v>2.39</v>
       </c>
       <c r="AP53" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ53">
         <v>33</v>
@@ -13995,7 +13995,7 @@
         <v>2.4</v>
       </c>
       <c r="BB53" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC53">
         <v>368</v>
@@ -14045,7 +14045,7 @@
     </row>
     <row r="54" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D54">
         <v>100</v>
@@ -14159,7 +14159,7 @@
         <v>2.92</v>
       </c>
       <c r="AP54" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ54">
         <v>31</v>
@@ -14195,7 +14195,7 @@
         <v>2.93</v>
       </c>
       <c r="BB54" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC54">
         <v>403</v>
@@ -14356,10 +14356,10 @@
         <v>174</v>
       </c>
       <c r="AO55" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP55" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ55">
         <v>33</v>
@@ -14368,7 +14368,7 @@
         <v>135</v>
       </c>
       <c r="AS55" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AT55" t="s">
         <v>177</v>
@@ -14386,7 +14386,7 @@
         <v>174</v>
       </c>
       <c r="BB55" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BD55" t="s">
         <v>135</v>
@@ -14538,7 +14538,7 @@
         <v>3.7699999999999999E-3</v>
       </c>
       <c r="AP56" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ56">
         <v>29</v>
@@ -14547,7 +14547,7 @@
         <v>135</v>
       </c>
       <c r="AS56" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AT56" t="s">
         <v>177</v>
@@ -14565,7 +14565,7 @@
         <v>174</v>
       </c>
       <c r="BB56" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BD56" t="s">
         <v>135</v>
@@ -14717,7 +14717,7 @@
         <v>7.2399999999999999E-3</v>
       </c>
       <c r="AP57" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ57">
         <v>30</v>
@@ -14726,7 +14726,7 @@
         <v>135</v>
       </c>
       <c r="AS57" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AT57" t="s">
         <v>177</v>
@@ -14744,7 +14744,7 @@
         <v>174</v>
       </c>
       <c r="BB57" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BD57" t="s">
         <v>135</v>
@@ -14896,7 +14896,7 @@
         <v>8.4600000000000005E-3</v>
       </c>
       <c r="AP58" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ58">
         <v>31</v>
@@ -14905,7 +14905,7 @@
         <v>135</v>
       </c>
       <c r="AS58" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AT58" t="s">
         <v>177</v>
@@ -14923,7 +14923,7 @@
         <v>174</v>
       </c>
       <c r="BB58" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BD58" t="s">
         <v>135</v>
@@ -15075,7 +15075,7 @@
         <v>1.1010000000000001E-2</v>
       </c>
       <c r="AP59" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ59" s="5">
         <v>32</v>
@@ -15084,7 +15084,7 @@
         <v>135</v>
       </c>
       <c r="AS59" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AT59" t="s">
         <v>177</v>
@@ -15105,7 +15105,7 @@
       </c>
       <c r="BA59" s="8"/>
       <c r="BB59" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BD59" t="s">
         <v>135</v>
@@ -15148,7 +15148,7 @@
     </row>
     <row r="60" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B60" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C60" s="12"/>
       <c r="D60" s="10">
@@ -15266,7 +15266,7 @@
         <v>0.40799999999999997</v>
       </c>
       <c r="AP60" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ60" s="10">
         <v>30</v>
@@ -15302,7 +15302,7 @@
         <v>0.35699999999999998</v>
       </c>
       <c r="BB60" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC60" s="10">
         <v>295</v>
@@ -15347,7 +15347,7 @@
     </row>
     <row r="61" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B61" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C61" s="12"/>
       <c r="D61" s="10">
@@ -15465,7 +15465,7 @@
         <v>0.96899999999999997</v>
       </c>
       <c r="AP61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ61" s="10">
         <v>30</v>
@@ -15501,7 +15501,7 @@
         <v>1.02</v>
       </c>
       <c r="BB61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC61" s="10">
         <v>325</v>
@@ -15546,7 +15546,7 @@
     </row>
     <row r="62" spans="2:70" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C62" s="12"/>
       <c r="D62" s="10">
@@ -15664,7 +15664,7 @@
         <v>1.7849999999999999</v>
       </c>
       <c r="AP62" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ62" s="10">
         <v>30</v>
@@ -15700,7 +15700,7 @@
         <v>1.7849999999999999</v>
       </c>
       <c r="BB62" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC62" s="10">
         <v>330</v>
@@ -15745,7 +15745,7 @@
     </row>
     <row r="63" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B63" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C63" s="12"/>
       <c r="D63" s="10">
@@ -15859,7 +15859,7 @@
         <v>1.988</v>
       </c>
       <c r="AP63" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ63" s="10">
         <v>28</v>
@@ -15895,7 +15895,7 @@
         <v>2.1920000000000002</v>
       </c>
       <c r="BB63" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC63" s="10">
         <v>345</v>
@@ -15940,7 +15940,7 @@
     </row>
     <row r="64" spans="2:70" x14ac:dyDescent="0.3">
       <c r="B64" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C64" s="12"/>
       <c r="D64" s="10">
@@ -16058,7 +16058,7 @@
         <v>2.5489999999999999</v>
       </c>
       <c r="AP64" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ64" s="10">
         <v>28</v>
@@ -16094,7 +16094,7 @@
         <v>2.7530000000000001</v>
       </c>
       <c r="BB64" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC64" s="10">
         <v>375</v>
@@ -16139,7 +16139,7 @@
     </row>
     <row r="65" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B65" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C65" s="12"/>
       <c r="D65" s="10">
@@ -16257,7 +16257,7 @@
         <v>2.4980000000000002</v>
       </c>
       <c r="AP65" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ65" s="10">
         <v>28</v>
@@ -16293,7 +16293,7 @@
         <v>2.702</v>
       </c>
       <c r="BB65" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC65" s="10">
         <v>375</v>
@@ -16338,7 +16338,7 @@
     </row>
     <row r="66" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B66" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C66" s="12"/>
       <c r="D66" s="10">
@@ -16456,7 +16456,7 @@
         <v>2.702</v>
       </c>
       <c r="AP66" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AQ66" s="10">
         <v>29</v>
@@ -16492,7 +16492,7 @@
         <v>2.9060000000000001</v>
       </c>
       <c r="BB66" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BC66" s="10">
         <v>390</v>
@@ -16652,10 +16652,10 @@
         <v>174</v>
       </c>
       <c r="AO67" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP67" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ67" s="5">
         <v>18</v>
@@ -16688,10 +16688,10 @@
         <v>174</v>
       </c>
       <c r="BA67" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB67" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC67" s="5">
         <v>321.5</v>
@@ -16706,7 +16706,7 @@
         <v>135</v>
       </c>
       <c r="BG67" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH67" s="5" t="s">
         <v>175</v>
@@ -16730,13 +16730,13 @@
         <v>135</v>
       </c>
       <c r="BO67" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP67" s="5" t="s">
         <v>135</v>
       </c>
       <c r="BQ67" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR67" s="5" t="s">
         <v>173</v>
@@ -16860,10 +16860,10 @@
         <v>174</v>
       </c>
       <c r="AO68" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP68" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ68">
         <v>20</v>
@@ -16896,10 +16896,10 @@
         <v>174</v>
       </c>
       <c r="BA68" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB68" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC68">
         <v>347.7</v>
@@ -16914,7 +16914,7 @@
         <v>135</v>
       </c>
       <c r="BG68" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH68" t="s">
         <v>175</v>
@@ -16938,13 +16938,13 @@
         <v>135</v>
       </c>
       <c r="BO68" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP68" t="s">
         <v>135</v>
       </c>
       <c r="BQ68" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR68" t="s">
         <v>173</v>
@@ -17066,10 +17066,10 @@
         <v>174</v>
       </c>
       <c r="AO69" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP69" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ69">
         <v>21</v>
@@ -17102,10 +17102,10 @@
         <v>174</v>
       </c>
       <c r="BA69" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB69" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC69">
         <v>381.8</v>
@@ -17120,7 +17120,7 @@
         <v>135</v>
       </c>
       <c r="BG69" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH69" t="s">
         <v>175</v>
@@ -17144,13 +17144,13 @@
         <v>135</v>
       </c>
       <c r="BO69" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP69" t="s">
         <v>135</v>
       </c>
       <c r="BQ69" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR69" t="s">
         <v>173</v>
@@ -17272,10 +17272,10 @@
         <v>174</v>
       </c>
       <c r="AO70" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP70" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ70">
         <v>22</v>
@@ -17308,10 +17308,10 @@
         <v>174</v>
       </c>
       <c r="BA70" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB70" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC70">
         <v>397.1</v>
@@ -17326,7 +17326,7 @@
         <v>135</v>
       </c>
       <c r="BG70" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH70" t="s">
         <v>175</v>
@@ -17350,13 +17350,13 @@
         <v>135</v>
       </c>
       <c r="BO70" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP70" t="s">
         <v>135</v>
       </c>
       <c r="BQ70" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR70" t="s">
         <v>173</v>
@@ -17478,10 +17478,10 @@
         <v>174</v>
       </c>
       <c r="AO71" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP71" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ71">
         <v>24</v>
@@ -17514,10 +17514,10 @@
         <v>174</v>
       </c>
       <c r="BA71" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB71" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC71">
         <v>446.8</v>
@@ -17532,7 +17532,7 @@
         <v>135</v>
       </c>
       <c r="BG71" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH71" t="s">
         <v>175</v>
@@ -17556,13 +17556,13 @@
         <v>135</v>
       </c>
       <c r="BO71" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP71" t="s">
         <v>135</v>
       </c>
       <c r="BQ71" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR71" t="s">
         <v>173</v>
@@ -17684,10 +17684,10 @@
         <v>174</v>
       </c>
       <c r="AO72" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP72" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ72">
         <v>24</v>
@@ -17720,10 +17720,10 @@
         <v>174</v>
       </c>
       <c r="BA72" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB72" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC72">
         <v>473.9</v>
@@ -17738,7 +17738,7 @@
         <v>135</v>
       </c>
       <c r="BG72" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH72" t="s">
         <v>175</v>
@@ -17762,13 +17762,13 @@
         <v>135</v>
       </c>
       <c r="BO72" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP72" t="s">
         <v>135</v>
       </c>
       <c r="BQ72" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR72" t="s">
         <v>173</v>
@@ -17890,10 +17890,10 @@
         <v>174</v>
       </c>
       <c r="AO73" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP73" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ73">
         <v>23</v>
@@ -17926,10 +17926,10 @@
         <v>174</v>
       </c>
       <c r="BA73" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB73" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC73">
         <v>446.3</v>
@@ -17944,7 +17944,7 @@
         <v>135</v>
       </c>
       <c r="BG73" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH73" t="s">
         <v>175</v>
@@ -17968,13 +17968,13 @@
         <v>135</v>
       </c>
       <c r="BO73" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP73" t="s">
         <v>135</v>
       </c>
       <c r="BQ73" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR73" t="s">
         <v>173</v>
@@ -18014,7 +18014,7 @@
         <v>135</v>
       </c>
       <c r="M74" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N74" t="s">
         <v>171</v>
@@ -18096,10 +18096,10 @@
         <v>174</v>
       </c>
       <c r="AO74" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP74" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ74" s="5">
         <v>37</v>
@@ -18129,7 +18129,7 @@
       </c>
       <c r="BA74" s="5"/>
       <c r="BB74" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC74" s="5"/>
       <c r="BD74" t="s">
@@ -18198,7 +18198,7 @@
         <v>135</v>
       </c>
       <c r="M75" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N75" t="s">
         <v>171</v>
@@ -18279,10 +18279,10 @@
         <v>174</v>
       </c>
       <c r="AO75" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP75" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ75">
         <v>37</v>
@@ -18309,7 +18309,7 @@
         <v>174</v>
       </c>
       <c r="BB75" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BD75" t="s">
         <v>135</v>
@@ -18368,7 +18368,7 @@
         <v>135</v>
       </c>
       <c r="M76" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N76" t="s">
         <v>171</v>
@@ -18449,10 +18449,10 @@
         <v>174</v>
       </c>
       <c r="AO76" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP76" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ76">
         <v>37</v>
@@ -18479,7 +18479,7 @@
         <v>174</v>
       </c>
       <c r="BB76" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BD76" t="s">
         <v>135</v>
@@ -18541,7 +18541,7 @@
         <v>135</v>
       </c>
       <c r="M77" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N77" t="s">
         <v>171</v>
@@ -18622,10 +18622,10 @@
         <v>174</v>
       </c>
       <c r="AO77" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP77" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ77">
         <v>37</v>
@@ -18652,7 +18652,7 @@
         <v>174</v>
       </c>
       <c r="BB77" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BD77" t="s">
         <v>135</v>
@@ -18681,7 +18681,7 @@
     </row>
     <row r="78" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B78" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C78" s="5"/>
       <c r="D78" s="5">
@@ -18796,10 +18796,10 @@
         <v>174</v>
       </c>
       <c r="AO78" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP78" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ78" s="5">
         <v>18</v>
@@ -18832,10 +18832,10 @@
         <v>174</v>
       </c>
       <c r="BA78" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB78" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC78" s="5">
         <v>321.5</v>
@@ -18850,7 +18850,7 @@
         <v>135</v>
       </c>
       <c r="BG78" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH78" s="5" t="s">
         <v>175</v>
@@ -18874,13 +18874,13 @@
         <v>135</v>
       </c>
       <c r="BO78" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP78" s="5" t="s">
         <v>135</v>
       </c>
       <c r="BQ78" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR78" s="5" t="s">
         <v>173</v>
@@ -18890,7 +18890,7 @@
     </row>
     <row r="79" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B79" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D79">
         <v>50</v>
@@ -19004,10 +19004,10 @@
         <v>174</v>
       </c>
       <c r="AO79" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP79" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ79">
         <v>20</v>
@@ -19040,10 +19040,10 @@
         <v>174</v>
       </c>
       <c r="BA79" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB79" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC79">
         <v>347.7</v>
@@ -19058,7 +19058,7 @@
         <v>135</v>
       </c>
       <c r="BG79" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH79" t="s">
         <v>175</v>
@@ -19082,13 +19082,13 @@
         <v>135</v>
       </c>
       <c r="BO79" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP79" t="s">
         <v>135</v>
       </c>
       <c r="BQ79" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR79" t="s">
         <v>173</v>
@@ -19096,7 +19096,7 @@
     </row>
     <row r="80" spans="1:72" x14ac:dyDescent="0.3">
       <c r="B80" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D80">
         <v>75</v>
@@ -19210,10 +19210,10 @@
         <v>174</v>
       </c>
       <c r="AO80" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP80" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ80">
         <v>21</v>
@@ -19246,10 +19246,10 @@
         <v>174</v>
       </c>
       <c r="BA80" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB80" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC80">
         <v>381.8</v>
@@ -19264,7 +19264,7 @@
         <v>135</v>
       </c>
       <c r="BG80" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH80" t="s">
         <v>175</v>
@@ -19288,13 +19288,13 @@
         <v>135</v>
       </c>
       <c r="BO80" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP80" t="s">
         <v>135</v>
       </c>
       <c r="BQ80" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR80" t="s">
         <v>173</v>
@@ -19302,7 +19302,7 @@
     </row>
     <row r="81" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B81" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D81">
         <v>85</v>
@@ -19416,10 +19416,10 @@
         <v>174</v>
       </c>
       <c r="AO81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP81" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ81">
         <v>22</v>
@@ -19452,10 +19452,10 @@
         <v>174</v>
       </c>
       <c r="BA81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB81" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC81">
         <v>397.1</v>
@@ -19470,7 +19470,7 @@
         <v>135</v>
       </c>
       <c r="BG81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH81" t="s">
         <v>175</v>
@@ -19494,13 +19494,13 @@
         <v>135</v>
       </c>
       <c r="BO81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP81" t="s">
         <v>135</v>
       </c>
       <c r="BQ81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR81" t="s">
         <v>173</v>
@@ -19508,7 +19508,7 @@
     </row>
     <row r="82" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B82" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D82">
         <v>100</v>
@@ -19622,10 +19622,10 @@
         <v>174</v>
       </c>
       <c r="AO82" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP82" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ82">
         <v>24</v>
@@ -19658,10 +19658,10 @@
         <v>174</v>
       </c>
       <c r="BA82" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB82" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC82">
         <v>446.8</v>
@@ -19676,7 +19676,7 @@
         <v>135</v>
       </c>
       <c r="BG82" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH82" t="s">
         <v>175</v>
@@ -19700,13 +19700,13 @@
         <v>135</v>
       </c>
       <c r="BO82" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP82" t="s">
         <v>135</v>
       </c>
       <c r="BQ82" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR82" t="s">
         <v>173</v>
@@ -19714,7 +19714,7 @@
     </row>
     <row r="83" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B83" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D83">
         <v>110</v>
@@ -19828,10 +19828,10 @@
         <v>174</v>
       </c>
       <c r="AO83" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP83" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ83">
         <v>24</v>
@@ -19864,10 +19864,10 @@
         <v>174</v>
       </c>
       <c r="BA83" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB83" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC83">
         <v>473.9</v>
@@ -19882,7 +19882,7 @@
         <v>135</v>
       </c>
       <c r="BG83" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH83" t="s">
         <v>175</v>
@@ -19906,13 +19906,13 @@
         <v>135</v>
       </c>
       <c r="BO83" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP83" t="s">
         <v>135</v>
       </c>
       <c r="BQ83" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR83" t="s">
         <v>173</v>
@@ -19920,7 +19920,7 @@
     </row>
     <row r="84" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B84" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D84">
         <v>100</v>
@@ -20034,10 +20034,10 @@
         <v>174</v>
       </c>
       <c r="AO84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP84" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ84">
         <v>23</v>
@@ -20070,10 +20070,10 @@
         <v>174</v>
       </c>
       <c r="BA84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB84" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC84">
         <v>446.3</v>
@@ -20088,7 +20088,7 @@
         <v>135</v>
       </c>
       <c r="BG84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH84" t="s">
         <v>175</v>
@@ -20112,13 +20112,13 @@
         <v>135</v>
       </c>
       <c r="BO84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP84" t="s">
         <v>135</v>
       </c>
       <c r="BQ84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR84" t="s">
         <v>173</v>
@@ -20126,7 +20126,7 @@
     </row>
     <row r="85" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B85" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D85" s="14">
         <v>15</v>
@@ -20180,7 +20180,7 @@
         <v>135</v>
       </c>
       <c r="U85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V85" t="s">
         <v>173</v>
@@ -20192,13 +20192,13 @@
         <v>174</v>
       </c>
       <c r="Y85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z85" t="s">
         <v>174</v>
       </c>
       <c r="AA85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB85" t="s">
         <v>174</v>
@@ -20240,10 +20240,10 @@
         <v>174</v>
       </c>
       <c r="AO85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP85" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ85" s="18">
         <v>30.5</v>
@@ -20264,37 +20264,37 @@
         <v>20</v>
       </c>
       <c r="AW85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX85" t="s">
         <v>174</v>
       </c>
       <c r="AY85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ85" t="s">
         <v>174</v>
       </c>
       <c r="BA85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB85" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD85" t="s">
         <v>135</v>
       </c>
       <c r="BE85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF85" t="s">
         <v>135</v>
       </c>
       <c r="BG85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH85" t="s">
         <v>175</v>
@@ -20306,25 +20306,25 @@
         <v>20</v>
       </c>
       <c r="BK85" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL85" t="s">
         <v>172</v>
       </c>
       <c r="BM85" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN85" t="s">
         <v>135</v>
       </c>
       <c r="BO85" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP85" t="s">
         <v>135</v>
       </c>
       <c r="BQ85" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR85" t="s">
         <v>173</v>
@@ -20333,7 +20333,7 @@
     <row r="86" spans="1:85" x14ac:dyDescent="0.3">
       <c r="A86" s="5"/>
       <c r="B86" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D86" s="17">
         <v>25</v>
@@ -20387,7 +20387,7 @@
         <v>135</v>
       </c>
       <c r="U86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V86" t="s">
         <v>173</v>
@@ -20399,13 +20399,13 @@
         <v>174</v>
       </c>
       <c r="Y86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z86" t="s">
         <v>174</v>
       </c>
       <c r="AA86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB86" t="s">
         <v>174</v>
@@ -20447,10 +20447,10 @@
         <v>174</v>
       </c>
       <c r="AO86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP86" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ86" s="19">
         <v>31</v>
@@ -20471,37 +20471,37 @@
         <v>20</v>
       </c>
       <c r="AW86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX86" t="s">
         <v>174</v>
       </c>
       <c r="AY86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ86" t="s">
         <v>174</v>
       </c>
       <c r="BA86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB86" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD86" t="s">
         <v>135</v>
       </c>
       <c r="BE86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF86" t="s">
         <v>135</v>
       </c>
       <c r="BG86" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH86" t="s">
         <v>175</v>
@@ -20513,25 +20513,25 @@
         <v>20</v>
       </c>
       <c r="BK86" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL86" t="s">
         <v>172</v>
       </c>
       <c r="BM86" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN86" t="s">
         <v>135</v>
       </c>
       <c r="BO86" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP86" t="s">
         <v>135</v>
       </c>
       <c r="BQ86" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR86" t="s">
         <v>173</v>
@@ -20540,7 +20540,7 @@
     <row r="87" spans="1:85" x14ac:dyDescent="0.3">
       <c r="A87" s="5"/>
       <c r="B87" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D87" s="14">
         <v>50</v>
@@ -20594,7 +20594,7 @@
         <v>135</v>
       </c>
       <c r="U87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V87" t="s">
         <v>173</v>
@@ -20606,13 +20606,13 @@
         <v>174</v>
       </c>
       <c r="Y87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z87" t="s">
         <v>174</v>
       </c>
       <c r="AA87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB87" t="s">
         <v>174</v>
@@ -20654,10 +20654,10 @@
         <v>174</v>
       </c>
       <c r="AO87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP87" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ87" s="18">
         <v>31</v>
@@ -20678,37 +20678,37 @@
         <v>20</v>
       </c>
       <c r="AW87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX87" t="s">
         <v>174</v>
       </c>
       <c r="AY87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ87" t="s">
         <v>174</v>
       </c>
       <c r="BA87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB87" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD87" t="s">
         <v>135</v>
       </c>
       <c r="BE87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF87" t="s">
         <v>135</v>
       </c>
       <c r="BG87" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH87" t="s">
         <v>175</v>
@@ -20720,25 +20720,25 @@
         <v>20</v>
       </c>
       <c r="BK87" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL87" t="s">
         <v>172</v>
       </c>
       <c r="BM87" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN87" t="s">
         <v>135</v>
       </c>
       <c r="BO87" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP87" t="s">
         <v>135</v>
       </c>
       <c r="BQ87" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR87" t="s">
         <v>173</v>
@@ -20760,7 +20760,7 @@
     </row>
     <row r="88" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B88" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D88" s="17">
         <v>75</v>
@@ -20814,7 +20814,7 @@
         <v>135</v>
       </c>
       <c r="U88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V88" t="s">
         <v>173</v>
@@ -20826,13 +20826,13 @@
         <v>174</v>
       </c>
       <c r="Y88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z88" t="s">
         <v>174</v>
       </c>
       <c r="AA88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB88" t="s">
         <v>174</v>
@@ -20874,10 +20874,10 @@
         <v>174</v>
       </c>
       <c r="AO88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP88" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ88" s="19">
         <v>32</v>
@@ -20898,37 +20898,37 @@
         <v>20</v>
       </c>
       <c r="AW88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX88" t="s">
         <v>174</v>
       </c>
       <c r="AY88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ88" t="s">
         <v>174</v>
       </c>
       <c r="BA88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB88" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD88" t="s">
         <v>135</v>
       </c>
       <c r="BE88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF88" t="s">
         <v>135</v>
       </c>
       <c r="BG88" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH88" t="s">
         <v>175</v>
@@ -20940,25 +20940,25 @@
         <v>20</v>
       </c>
       <c r="BK88" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL88" t="s">
         <v>172</v>
       </c>
       <c r="BM88" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN88" t="s">
         <v>135</v>
       </c>
       <c r="BO88" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP88" t="s">
         <v>135</v>
       </c>
       <c r="BQ88" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR88" t="s">
         <v>173</v>
@@ -20966,7 +20966,7 @@
     </row>
     <row r="89" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B89" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D89" s="14">
         <v>85</v>
@@ -21020,7 +21020,7 @@
         <v>135</v>
       </c>
       <c r="U89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V89" t="s">
         <v>173</v>
@@ -21032,13 +21032,13 @@
         <v>174</v>
       </c>
       <c r="Y89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z89" t="s">
         <v>174</v>
       </c>
       <c r="AA89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB89" t="s">
         <v>174</v>
@@ -21080,10 +21080,10 @@
         <v>174</v>
       </c>
       <c r="AO89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP89" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ89" s="18">
         <v>32.5</v>
@@ -21104,37 +21104,37 @@
         <v>20</v>
       </c>
       <c r="AW89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX89" t="s">
         <v>174</v>
       </c>
       <c r="AY89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ89" t="s">
         <v>174</v>
       </c>
       <c r="BA89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB89" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD89" t="s">
         <v>135</v>
       </c>
       <c r="BE89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF89" t="s">
         <v>135</v>
       </c>
       <c r="BG89" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH89" t="s">
         <v>175</v>
@@ -21146,25 +21146,25 @@
         <v>20</v>
       </c>
       <c r="BK89" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL89" t="s">
         <v>172</v>
       </c>
       <c r="BM89" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN89" t="s">
         <v>135</v>
       </c>
       <c r="BO89" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP89" t="s">
         <v>135</v>
       </c>
       <c r="BQ89" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR89" t="s">
         <v>173</v>
@@ -21172,7 +21172,7 @@
     </row>
     <row r="90" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B90" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D90" s="17">
         <v>90</v>
@@ -21226,7 +21226,7 @@
         <v>135</v>
       </c>
       <c r="U90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V90" t="s">
         <v>173</v>
@@ -21238,13 +21238,13 @@
         <v>174</v>
       </c>
       <c r="Y90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z90" t="s">
         <v>174</v>
       </c>
       <c r="AA90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB90" t="s">
         <v>174</v>
@@ -21286,10 +21286,10 @@
         <v>174</v>
       </c>
       <c r="AO90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP90" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ90" s="19">
         <v>32.5</v>
@@ -21310,37 +21310,37 @@
         <v>20</v>
       </c>
       <c r="AW90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX90" t="s">
         <v>174</v>
       </c>
       <c r="AY90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ90" t="s">
         <v>174</v>
       </c>
       <c r="BA90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB90" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD90" t="s">
         <v>135</v>
       </c>
       <c r="BE90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF90" t="s">
         <v>135</v>
       </c>
       <c r="BG90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH90" t="s">
         <v>175</v>
@@ -21352,25 +21352,25 @@
         <v>20</v>
       </c>
       <c r="BK90" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL90" t="s">
         <v>172</v>
       </c>
       <c r="BM90" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN90" t="s">
         <v>135</v>
       </c>
       <c r="BO90" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP90" t="s">
         <v>135</v>
       </c>
       <c r="BQ90" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR90" t="s">
         <v>173</v>
@@ -21378,7 +21378,7 @@
     </row>
     <row r="91" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B91" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C91" s="5"/>
       <c r="D91" s="14">
@@ -21433,7 +21433,7 @@
         <v>135</v>
       </c>
       <c r="U91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V91" t="s">
         <v>173</v>
@@ -21445,13 +21445,13 @@
         <v>174</v>
       </c>
       <c r="Y91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z91" t="s">
         <v>174</v>
       </c>
       <c r="AA91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB91" t="s">
         <v>174</v>
@@ -21493,10 +21493,10 @@
         <v>174</v>
       </c>
       <c r="AO91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP91" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ91" s="18">
         <v>33</v>
@@ -21517,37 +21517,37 @@
         <v>20</v>
       </c>
       <c r="AW91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX91" t="s">
         <v>174</v>
       </c>
       <c r="AY91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ91" t="s">
         <v>174</v>
       </c>
       <c r="BA91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB91" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD91" t="s">
         <v>135</v>
       </c>
       <c r="BE91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF91" t="s">
         <v>135</v>
       </c>
       <c r="BG91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH91" t="s">
         <v>175</v>
@@ -21559,25 +21559,25 @@
         <v>20</v>
       </c>
       <c r="BK91" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL91" t="s">
         <v>172</v>
       </c>
       <c r="BM91" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN91" t="s">
         <v>135</v>
       </c>
       <c r="BO91" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP91" t="s">
         <v>135</v>
       </c>
       <c r="BQ91" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR91" t="s">
         <v>173</v>
@@ -21586,7 +21586,7 @@
     </row>
     <row r="92" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B92" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D92" s="17">
         <v>100</v>
@@ -21640,7 +21640,7 @@
         <v>135</v>
       </c>
       <c r="U92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V92" t="s">
         <v>173</v>
@@ -21652,13 +21652,13 @@
         <v>174</v>
       </c>
       <c r="Y92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z92" t="s">
         <v>174</v>
       </c>
       <c r="AA92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB92" t="s">
         <v>174</v>
@@ -21700,10 +21700,10 @@
         <v>174</v>
       </c>
       <c r="AO92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP92" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ92" s="19">
         <v>33</v>
@@ -21724,37 +21724,37 @@
         <v>20</v>
       </c>
       <c r="AW92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX92" t="s">
         <v>174</v>
       </c>
       <c r="AY92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ92" t="s">
         <v>174</v>
       </c>
       <c r="BA92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB92" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD92" t="s">
         <v>135</v>
       </c>
       <c r="BE92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF92" t="s">
         <v>135</v>
       </c>
       <c r="BG92" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH92" t="s">
         <v>175</v>
@@ -21766,25 +21766,25 @@
         <v>20</v>
       </c>
       <c r="BK92" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL92" t="s">
         <v>172</v>
       </c>
       <c r="BM92" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN92" t="s">
         <v>135</v>
       </c>
       <c r="BO92" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP92" t="s">
         <v>135</v>
       </c>
       <c r="BQ92" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR92" t="s">
         <v>173</v>
@@ -21792,7 +21792,7 @@
     </row>
     <row r="93" spans="1:85" x14ac:dyDescent="0.3">
       <c r="B93" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D93" s="14">
         <v>110</v>
@@ -21846,7 +21846,7 @@
         <v>135</v>
       </c>
       <c r="U93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="V93" t="s">
         <v>173</v>
@@ -21858,13 +21858,13 @@
         <v>174</v>
       </c>
       <c r="Y93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Z93" t="s">
         <v>174</v>
       </c>
       <c r="AA93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AB93" t="s">
         <v>174</v>
@@ -21906,10 +21906,10 @@
         <v>174</v>
       </c>
       <c r="AO93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AP93" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ93" s="18">
         <v>32.5</v>
@@ -21930,37 +21930,37 @@
         <v>20</v>
       </c>
       <c r="AW93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AX93" t="s">
         <v>174</v>
       </c>
       <c r="AY93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AZ93" t="s">
         <v>174</v>
       </c>
       <c r="BA93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BB93" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BC93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BD93" t="s">
         <v>135</v>
       </c>
       <c r="BE93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BF93" t="s">
         <v>135</v>
       </c>
       <c r="BG93" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BH93" t="s">
         <v>175</v>
@@ -21972,25 +21972,25 @@
         <v>20</v>
       </c>
       <c r="BK93" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BL93" t="s">
         <v>172</v>
       </c>
       <c r="BM93" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BN93" t="s">
         <v>135</v>
       </c>
       <c r="BO93" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BP93" t="s">
         <v>135</v>
       </c>
       <c r="BQ93" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="BR93" t="s">
         <v>173</v>

</xml_diff>